<commit_message>
Add bill_to_3 to CI Shipping Mark and update templates
CI generator now writes bill_to_3 to A32 (matching PL pattern).
Updated CI/FI/PL Excel templates and documentation.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/commercial_invoice.xlsx
+++ b/templates/commercial_invoice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rotork-my.sharepoint.com/personal/jeongtaek_bang_rotork_com/Documents/바탕 화면/업무/NOAH ACTUATION/noahAutomation/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_482B29FEF0C7F80AEE82E0F7E4E761DFCF1F255D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12301E47-9A3A-4006-B8DB-C355D22F84BA}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="11_482B29FEF0C7F80AEE82E0F7E4E761DFCF1F255D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F09190C3-E9AF-46D7-B03F-37F391EF987C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="51">
   <si>
     <t>Commercial Invoice</t>
   </si>
@@ -193,6 +193,10 @@
   </si>
   <si>
     <t>www.rotork.com/en/terms-and-conditions/customers</t>
+  </si>
+  <si>
+    <t>INCOTERMS</t>
+    <phoneticPr fontId="17" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -801,13 +805,13 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>132522</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>12906</xdr:rowOff>
+      <xdr:rowOff>21261</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>667441</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>322743</xdr:rowOff>
+      <xdr:rowOff>331098</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -830,8 +834,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="132522" y="12906"/>
-          <a:ext cx="1454289" cy="906185"/>
+          <a:off x="132522" y="21261"/>
+          <a:ext cx="1462353" cy="911416"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -852,7 +856,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>750374</xdr:colOff>
+      <xdr:colOff>608335</xdr:colOff>
       <xdr:row>36</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -1191,8 +1195,8 @@
     <col min="3" max="3" width="13.83203125" style="44" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6.6640625" style="44" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.33203125" style="44" customWidth="1"/>
-    <col min="6" max="6" width="12" style="44" customWidth="1"/>
-    <col min="7" max="7" width="14.33203125" style="44" customWidth="1"/>
+    <col min="6" max="6" width="16.1640625" style="44" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" style="44" customWidth="1"/>
     <col min="8" max="8" width="9" style="44" customWidth="1"/>
     <col min="9" max="9" width="14.33203125" style="44" customWidth="1"/>
     <col min="10" max="10" width="14" style="44" customWidth="1"/>
@@ -1468,7 +1472,9 @@
       <c r="C18" s="51"/>
       <c r="D18" s="51"/>
       <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
+      <c r="F18" s="3" t="s">
+        <v>50</v>
+      </c>
       <c r="G18" s="3" t="s">
         <v>29</v>
       </c>
@@ -1926,7 +1932,7 @@
   <hyperlinks>
     <hyperlink ref="F41" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.59055118110236227" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
   <drawing r:id="rId3"/>
 </worksheet>

</xml_diff>

<commit_message>
Rename AX Project number to Model code, update DN PKs, remove GL대상 logic
- Rename [AX Project number] → [Model code] across Power Query formulas and docs
- Remove GL대상 flag logic from DN_원가포함 query (no longer needed)
- Add ReplaceErrorValues to all Power Query sources for robust error handling
- Update DN PK to (DN_ID, SO_ID, Line item) in db_schema and docs
- Update .gitignore with generated_pi/fi, temp files, data files
- Update CI/FI/OC/PL Excel templates

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/commercial_invoice.xlsx
+++ b/templates/commercial_invoice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rotork-my.sharepoint.com/personal/jeongtaek_bang_rotork_com/Documents/바탕 화면/업무/NOAH ACTUATION/noahAutomation/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="11_482B29FEF0C7F80AEE82E0F7E4E761DFCF1F255D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F09190C3-E9AF-46D7-B03F-37F391EF987C}"/>
+  <xr:revisionPtr revIDLastSave="84" documentId="11_482B29FEF0C7F80AEE82E0F7E4E761DFCF1F255D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{642D3CBD-35D9-4568-811B-D2C4B4C6954C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,8 +16,8 @@
     <sheet name="Table 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Table 1'!$A$1:$I$41</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Table 1'!$1:$17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Table 1'!$A$1:$I$42</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Table 1'!$1:$18</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="47">
   <si>
     <t>Commercial Invoice</t>
   </si>
@@ -51,25 +51,10 @@
     <t>Date:</t>
   </si>
   <si>
-    <t>515, 5th floor Leader’s Bldg, Jangmi-ro 42,</t>
-  </si>
-  <si>
-    <t>L/C No:</t>
-  </si>
-  <si>
-    <t>Bundang-gu, Seongnam-si, Gyeonggi-do, 13496, Korea</t>
-  </si>
-  <si>
     <t>Applicant(If other than consignee)</t>
   </si>
   <si>
-    <t>Tel : 82-31-768-8151  Fax: 82-31-768-8156</t>
-  </si>
-  <si>
     <t>Consigned to :</t>
-  </si>
-  <si>
-    <t>ASC Engineered Solutions 2001 Spring Road Suite 300 Oak Brook, IL 60523</t>
   </si>
   <si>
     <t xml:space="preserve">Vessel  Name or Flight No
@@ -79,9 +64,6 @@
     <t>Other reference :</t>
   </si>
   <si>
-    <t xml:space="preserve">HS CODE : </t>
-  </si>
-  <si>
     <t>8481.90.3000</t>
   </si>
   <si>
@@ -126,9 +108,6 @@
   </si>
   <si>
     <t>Electric Actuator</t>
-  </si>
-  <si>
-    <t>EX-WORKS</t>
   </si>
   <si>
     <t>5350008920 BUSHING 17STAR FOR ABZ015/019</t>
@@ -195,7 +174,21 @@
     <t>www.rotork.com/en/terms-and-conditions/customers</t>
   </si>
   <si>
-    <t>INCOTERMS</t>
+    <t>Payment terms:</t>
+    <phoneticPr fontId="17" type="noConversion"/>
+  </si>
+  <si>
+    <t>Incoterms:</t>
+    <phoneticPr fontId="17" type="noConversion"/>
+  </si>
+  <si>
+    <t>515, 5th floor Leader’s Bldg, Jangmi-ro 42,
+Bundang-gu, Seongnam-si, Gyeonggi-do, 13496, Korea
+Tel : 82-31-768-8151  Fax: 82-31-768-8156</t>
+    <phoneticPr fontId="17" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">HS CODE: </t>
     <phoneticPr fontId="17" type="noConversion"/>
   </si>
 </sst>
@@ -537,7 +530,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -553,9 +546,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -604,9 +594,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -627,9 +614,6 @@
     </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -677,10 +661,20 @@
     <xf numFmtId="178" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" indent="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -689,33 +683,39 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
@@ -726,12 +726,17 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -748,35 +753,44 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma [0]" xfId="2" builtinId="6"/>
@@ -851,13 +865,13 @@
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>31</xdr:row>
+      <xdr:row>32</xdr:row>
       <xdr:rowOff>160141</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>608335</xdr:colOff>
-      <xdr:row>36</xdr:row>
+      <xdr:colOff>783796</xdr:colOff>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1187,31 +1201,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J42"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.5" style="44" customWidth="1"/>
-    <col min="2" max="2" width="5.6640625" style="44" customWidth="1"/>
-    <col min="3" max="3" width="13.83203125" style="44" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.6640625" style="44" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.33203125" style="44" customWidth="1"/>
-    <col min="6" max="6" width="16.1640625" style="44" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" style="44" customWidth="1"/>
-    <col min="8" max="8" width="9" style="44" customWidth="1"/>
-    <col min="9" max="9" width="14.33203125" style="44" customWidth="1"/>
-    <col min="10" max="10" width="14" style="44" customWidth="1"/>
+    <col min="1" max="1" width="10.5" style="41" customWidth="1"/>
+    <col min="2" max="2" width="5.6640625" style="41" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" style="41" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.33203125" style="41" customWidth="1"/>
+    <col min="5" max="5" width="9.5" style="41" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" style="41" customWidth="1"/>
+    <col min="7" max="7" width="11.6640625" style="41" customWidth="1"/>
+    <col min="8" max="8" width="11.1640625" style="41" customWidth="1"/>
+    <col min="9" max="9" width="24.5" style="41" customWidth="1"/>
+    <col min="10" max="10" width="14" style="41" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="78"/>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
+      <c r="A1" s="45"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1219,12 +1233,12 @@
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
-      <c r="E2" s="80" t="s">
+      <c r="E2" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
     </row>
@@ -1241,698 +1255,700 @@
       <c r="J3" s="2"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="50" t="s">
+      <c r="A4" s="51" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="51"/>
-      <c r="C4" s="51"/>
-      <c r="D4" s="51"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="33" t="s">
+      <c r="B4" s="52"/>
+      <c r="C4" s="52"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="G4" s="32"/>
-      <c r="H4" s="20" t="s">
+      <c r="G4" s="29"/>
+      <c r="H4" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="32"/>
+      <c r="I4" s="29"/>
       <c r="J4" s="1"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="83" t="s">
+    <row r="5" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="61" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="90"/>
+      <c r="C5" s="90"/>
+      <c r="D5" s="90"/>
+      <c r="E5" s="91"/>
+      <c r="F5" s="44" t="s">
+        <v>44</v>
+      </c>
+      <c r="G5" s="25"/>
+      <c r="H5" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="I5" s="25"/>
+      <c r="J5" s="1"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" s="92"/>
+      <c r="B6" s="90"/>
+      <c r="C6" s="90"/>
+      <c r="D6" s="90"/>
+      <c r="E6" s="91"/>
+      <c r="F6" s="60" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="48"/>
-      <c r="C5" s="48"/>
-      <c r="D5" s="48"/>
-      <c r="E5" s="54"/>
-      <c r="F5" s="33" t="s">
+      <c r="G6" s="52"/>
+      <c r="H6" s="52"/>
+      <c r="I6" s="53"/>
+      <c r="J6" s="1"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" s="93"/>
+      <c r="B7" s="94"/>
+      <c r="C7" s="94"/>
+      <c r="D7" s="94"/>
+      <c r="E7" s="95"/>
+      <c r="F7" s="83"/>
+      <c r="G7" s="46"/>
+      <c r="H7" s="46"/>
+      <c r="I7" s="75"/>
+      <c r="J7" s="1"/>
+    </row>
+    <row r="8" spans="1:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="51" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="27"/>
-      <c r="H5" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="I5" s="27"/>
-      <c r="J5" s="1"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="83" t="s">
+      <c r="B8" s="52"/>
+      <c r="C8" s="52"/>
+      <c r="D8" s="52"/>
+      <c r="E8" s="53"/>
+      <c r="F8" s="84"/>
+      <c r="G8" s="46"/>
+      <c r="H8" s="46"/>
+      <c r="I8" s="75"/>
+      <c r="J8" s="1"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9" s="61"/>
+      <c r="B9" s="62"/>
+      <c r="C9" s="62"/>
+      <c r="D9" s="62"/>
+      <c r="E9" s="63"/>
+      <c r="F9" s="84"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="46"/>
+      <c r="I9" s="75"/>
+      <c r="J9" s="4"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" s="61"/>
+      <c r="B10" s="62"/>
+      <c r="C10" s="62"/>
+      <c r="D10" s="62"/>
+      <c r="E10" s="63"/>
+      <c r="F10" s="84"/>
+      <c r="G10" s="46"/>
+      <c r="H10" s="46"/>
+      <c r="I10" s="75"/>
+      <c r="J10" s="4"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11" s="64"/>
+      <c r="B11" s="65"/>
+      <c r="C11" s="65"/>
+      <c r="D11" s="65"/>
+      <c r="E11" s="66"/>
+      <c r="F11" s="85"/>
+      <c r="G11" s="57"/>
+      <c r="H11" s="57"/>
+      <c r="I11" s="48"/>
+      <c r="J11" s="2"/>
+    </row>
+    <row r="12" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="48"/>
-      <c r="C6" s="48"/>
-      <c r="D6" s="48"/>
-      <c r="E6" s="54"/>
-      <c r="F6" s="62" t="s">
+      <c r="B12" s="52"/>
+      <c r="C12" s="52"/>
+      <c r="D12" s="52"/>
+      <c r="E12" s="53"/>
+      <c r="F12" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="51"/>
-      <c r="H6" s="51"/>
-      <c r="I6" s="52"/>
-      <c r="J6" s="1"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="85" t="s">
+      <c r="G12" s="53"/>
+      <c r="H12" s="87" t="s">
+        <v>46</v>
+      </c>
+      <c r="I12" s="86" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="57"/>
-      <c r="C7" s="57"/>
-      <c r="D7" s="57"/>
-      <c r="E7" s="58"/>
-      <c r="F7" s="53"/>
-      <c r="G7" s="48"/>
-      <c r="H7" s="48"/>
-      <c r="I7" s="54"/>
-      <c r="J7" s="1"/>
-    </row>
-    <row r="8" spans="1:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="50" t="s">
+      <c r="J12" s="2"/>
+    </row>
+    <row r="13" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="56"/>
+      <c r="B13" s="57"/>
+      <c r="C13" s="57"/>
+      <c r="D13" s="57"/>
+      <c r="E13" s="48"/>
+      <c r="F13" s="84"/>
+      <c r="G13" s="75"/>
+      <c r="H13" s="46"/>
+      <c r="I13" s="75"/>
+      <c r="J13" s="2"/>
+    </row>
+    <row r="14" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="51"/>
-      <c r="C8" s="51"/>
-      <c r="D8" s="51"/>
-      <c r="E8" s="52"/>
-      <c r="F8" s="55"/>
-      <c r="G8" s="48"/>
-      <c r="H8" s="48"/>
-      <c r="I8" s="54"/>
-      <c r="J8" s="1"/>
-    </row>
-    <row r="9" spans="1:10" ht="33.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="84" t="s">
+      <c r="B14" s="70" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="48"/>
-      <c r="C9" s="48"/>
-      <c r="D9" s="48"/>
-      <c r="E9" s="54"/>
-      <c r="F9" s="55"/>
-      <c r="G9" s="48"/>
-      <c r="H9" s="48"/>
-      <c r="I9" s="54"/>
-      <c r="J9" s="4"/>
-    </row>
-    <row r="10" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="30"/>
-      <c r="B10" s="22"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="56"/>
-      <c r="G10" s="57"/>
-      <c r="H10" s="57"/>
-      <c r="I10" s="58"/>
-      <c r="J10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="50" t="s">
+      <c r="C14" s="71"/>
+      <c r="D14" s="71"/>
+      <c r="E14" s="69"/>
+      <c r="F14" s="74" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="51"/>
-      <c r="C11" s="51"/>
-      <c r="D11" s="51"/>
-      <c r="E11" s="52"/>
-      <c r="F11" s="62" t="s">
+      <c r="G14" s="75"/>
+      <c r="H14" s="46"/>
+      <c r="I14" s="75"/>
+      <c r="J14" s="2"/>
+    </row>
+    <row r="15" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="G11" s="52"/>
-      <c r="H11" s="61" t="s">
-        <v>13</v>
-      </c>
-      <c r="I11" s="59" t="s">
+      <c r="B15" s="70"/>
+      <c r="C15" s="71"/>
+      <c r="D15" s="71"/>
+      <c r="E15" s="69"/>
+      <c r="F15" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="J11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="86"/>
-      <c r="B12" s="57"/>
-      <c r="C12" s="57"/>
-      <c r="D12" s="57"/>
-      <c r="E12" s="58"/>
-      <c r="F12" s="55"/>
-      <c r="G12" s="54"/>
-      <c r="H12" s="48"/>
-      <c r="I12" s="54"/>
-      <c r="J12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="34" t="s">
+      <c r="G15" s="48"/>
+      <c r="H15" s="57"/>
+      <c r="I15" s="48"/>
+      <c r="J15" s="2"/>
+    </row>
+    <row r="16" spans="1:10" ht="17.850000000000001" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="76" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="69" t="s">
+      <c r="B16" s="71"/>
+      <c r="C16" s="71"/>
+      <c r="D16" s="68">
+        <v>46030</v>
+      </c>
+      <c r="E16" s="69"/>
+      <c r="F16" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="65"/>
-      <c r="D13" s="65"/>
-      <c r="E13" s="68"/>
-      <c r="F13" s="71" t="s">
+      <c r="G16" s="20"/>
+      <c r="H16" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="G13" s="54"/>
-      <c r="H13" s="48"/>
-      <c r="I13" s="54"/>
-      <c r="J13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="34" t="s">
+      <c r="I16" s="27"/>
+      <c r="J16" s="1"/>
+    </row>
+    <row r="17" spans="1:10" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="33"/>
+      <c r="B17" s="33"/>
+      <c r="C17" s="33"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="34"/>
+      <c r="F17" s="35"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="36"/>
+      <c r="I17" s="37"/>
+      <c r="J17" s="1"/>
+    </row>
+    <row r="18" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="89" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="69"/>
-      <c r="C14" s="65"/>
-      <c r="D14" s="65"/>
-      <c r="E14" s="68"/>
-      <c r="F14" s="79" t="s">
+      <c r="B18" s="71"/>
+      <c r="C18" s="71"/>
+      <c r="D18" s="71"/>
+      <c r="E18" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F18" s="40"/>
+      <c r="G18" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="G14" s="58"/>
-      <c r="H14" s="57"/>
-      <c r="I14" s="58"/>
-      <c r="J14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" ht="17.850000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="72" t="s">
+      <c r="H18" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="65"/>
-      <c r="C15" s="65"/>
-      <c r="D15" s="67">
-        <v>46030</v>
-      </c>
-      <c r="E15" s="68"/>
-      <c r="F15" s="26" t="s">
+      <c r="I18" s="39"/>
+      <c r="J18" s="11"/>
+    </row>
+    <row r="19" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="77" t="s">
         <v>22</v>
       </c>
-      <c r="G15" s="21"/>
-      <c r="H15" s="24" t="s">
+      <c r="B19" s="52"/>
+      <c r="C19" s="52"/>
+      <c r="D19" s="52"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="16"/>
+      <c r="I19" s="16"/>
+      <c r="J19" s="1"/>
+    </row>
+    <row r="20" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="73" t="s">
         <v>23</v>
       </c>
-      <c r="I15" s="29"/>
-      <c r="J15" s="1"/>
-    </row>
-    <row r="16" spans="1:10" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="36"/>
-      <c r="B16" s="36"/>
-      <c r="C16" s="36"/>
-      <c r="D16" s="41"/>
-      <c r="E16" s="37"/>
-      <c r="F16" s="38"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="39"/>
-      <c r="I16" s="40"/>
-      <c r="J16" s="1"/>
-    </row>
-    <row r="17" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="64" t="s">
+      <c r="B20" s="46"/>
+      <c r="C20" s="46"/>
+      <c r="D20" s="46"/>
+      <c r="E20" s="6">
+        <v>10</v>
+      </c>
+      <c r="F20" s="1"/>
+      <c r="G20" s="42">
         <v>24</v>
       </c>
-      <c r="B17" s="65"/>
-      <c r="C17" s="65"/>
-      <c r="D17" s="65"/>
-      <c r="E17" s="42" t="s">
+      <c r="H20" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="I20" s="7">
+        <f t="shared" ref="I20:I27" si="0">E20*G20</f>
+        <v>240</v>
+      </c>
+      <c r="J20" s="1"/>
+    </row>
+    <row r="21" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="73" t="s">
         <v>25</v>
       </c>
-      <c r="F17" s="43"/>
-      <c r="G17" s="42" t="s">
-        <v>26</v>
-      </c>
-      <c r="H17" s="42" t="s">
-        <v>27</v>
-      </c>
-      <c r="I17" s="42"/>
-      <c r="J17" s="12"/>
-    </row>
-    <row r="18" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="73" t="s">
-        <v>28</v>
-      </c>
-      <c r="B18" s="51"/>
-      <c r="C18" s="51"/>
-      <c r="D18" s="51"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="H18" s="17"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="1"/>
-    </row>
-    <row r="19" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="60" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19" s="48"/>
-      <c r="C19" s="48"/>
-      <c r="D19" s="48"/>
-      <c r="E19" s="7">
+      <c r="B21" s="46"/>
+      <c r="C21" s="46"/>
+      <c r="D21" s="46"/>
+      <c r="E21" s="6">
         <v>10</v>
       </c>
-      <c r="F19" s="1"/>
-      <c r="G19" s="45">
+      <c r="F21" s="1"/>
+      <c r="G21" s="42">
+        <v>1.26</v>
+      </c>
+      <c r="H21" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="H19" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="I19" s="8">
-        <f t="shared" ref="I19:I26" si="0">E19*G19</f>
-        <v>240</v>
-      </c>
-      <c r="J19" s="1"/>
-    </row>
-    <row r="20" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="60" t="s">
-        <v>32</v>
-      </c>
-      <c r="B20" s="48"/>
-      <c r="C20" s="48"/>
-      <c r="D20" s="48"/>
-      <c r="E20" s="7">
-        <v>10</v>
-      </c>
-      <c r="F20" s="1"/>
-      <c r="G20" s="45">
-        <v>1.26</v>
-      </c>
-      <c r="H20" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="I20" s="8">
+      <c r="I21" s="7">
         <f t="shared" si="0"/>
         <v>12.6</v>
       </c>
-      <c r="J20" s="1"/>
-    </row>
-    <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="B21" s="48"/>
-      <c r="C21" s="48"/>
-      <c r="D21" s="48"/>
-      <c r="E21" s="7">
+      <c r="J21" s="1"/>
+    </row>
+    <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="73" t="s">
+        <v>26</v>
+      </c>
+      <c r="B22" s="46"/>
+      <c r="C22" s="46"/>
+      <c r="D22" s="46"/>
+      <c r="E22" s="6">
         <v>10</v>
       </c>
-      <c r="F21" s="1"/>
-      <c r="G21" s="45">
+      <c r="F22" s="1"/>
+      <c r="G22" s="42">
         <v>3.7</v>
       </c>
-      <c r="H21" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="I21" s="8">
+      <c r="H22" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="I22" s="7">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="J21" s="1"/>
-    </row>
-    <row r="22" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="60" t="s">
-        <v>34</v>
-      </c>
-      <c r="B22" s="48"/>
-      <c r="C22" s="48"/>
-      <c r="D22" s="48"/>
-      <c r="E22" s="7">
+      <c r="J22" s="1"/>
+    </row>
+    <row r="23" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="73" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" s="46"/>
+      <c r="C23" s="46"/>
+      <c r="D23" s="46"/>
+      <c r="E23" s="6">
         <v>10</v>
       </c>
-      <c r="F22" s="1"/>
-      <c r="G22" s="45">
+      <c r="F23" s="1"/>
+      <c r="G23" s="42">
         <v>3.9</v>
       </c>
-      <c r="H22" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="I22" s="8">
+      <c r="H23" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="I23" s="7">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
-      <c r="J22" s="1"/>
-    </row>
-    <row r="23" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="60" t="s">
-        <v>35</v>
-      </c>
-      <c r="B23" s="48"/>
-      <c r="C23" s="48"/>
-      <c r="D23" s="48"/>
-      <c r="E23" s="7">
+      <c r="J23" s="1"/>
+    </row>
+    <row r="24" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="73" t="s">
+        <v>28</v>
+      </c>
+      <c r="B24" s="46"/>
+      <c r="C24" s="46"/>
+      <c r="D24" s="46"/>
+      <c r="E24" s="6">
         <v>10</v>
       </c>
-      <c r="F23" s="1"/>
-      <c r="G23" s="45">
+      <c r="F24" s="1"/>
+      <c r="G24" s="42">
         <v>3.9</v>
       </c>
-      <c r="H23" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="I23" s="8">
+      <c r="H24" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="I24" s="7">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
-      <c r="J23" s="1"/>
-    </row>
-    <row r="24" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="60" t="s">
-        <v>36</v>
-      </c>
-      <c r="B24" s="48"/>
-      <c r="C24" s="48"/>
-      <c r="D24" s="48"/>
-      <c r="E24" s="7">
+      <c r="J24" s="1"/>
+    </row>
+    <row r="25" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="73" t="s">
+        <v>29</v>
+      </c>
+      <c r="B25" s="46"/>
+      <c r="C25" s="46"/>
+      <c r="D25" s="46"/>
+      <c r="E25" s="6">
         <v>10</v>
       </c>
-      <c r="F24" s="1"/>
-      <c r="G24" s="45">
+      <c r="F25" s="1"/>
+      <c r="G25" s="42">
         <v>2.5</v>
       </c>
-      <c r="H24" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="I24" s="8">
+      <c r="H25" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="I25" s="7">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="J24" s="1"/>
-    </row>
-    <row r="25" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="60" t="s">
-        <v>37</v>
-      </c>
-      <c r="B25" s="48"/>
-      <c r="C25" s="48"/>
-      <c r="D25" s="48"/>
-      <c r="E25" s="7">
+      <c r="J25" s="1"/>
+    </row>
+    <row r="26" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="73" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26" s="46"/>
+      <c r="C26" s="46"/>
+      <c r="D26" s="46"/>
+      <c r="E26" s="6">
         <v>10</v>
       </c>
-      <c r="F25" s="1"/>
-      <c r="G25" s="45">
+      <c r="F26" s="1"/>
+      <c r="G26" s="42">
         <v>2.9</v>
       </c>
-      <c r="H25" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="I25" s="8">
+      <c r="H26" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="I26" s="7">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="J25" s="1"/>
-    </row>
-    <row r="26" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="70" t="s">
-        <v>38</v>
-      </c>
-      <c r="B26" s="57"/>
-      <c r="C26" s="57"/>
-      <c r="D26" s="57"/>
-      <c r="E26" s="9">
+      <c r="J26" s="1"/>
+    </row>
+    <row r="27" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="72" t="s">
+        <v>31</v>
+      </c>
+      <c r="B27" s="57"/>
+      <c r="C27" s="57"/>
+      <c r="D27" s="57"/>
+      <c r="E27" s="8">
         <v>10</v>
       </c>
-      <c r="F26" s="10"/>
-      <c r="G26" s="46">
+      <c r="F27" s="9"/>
+      <c r="G27" s="43">
         <v>2.9</v>
       </c>
-      <c r="H26" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="I26" s="8">
+      <c r="H27" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="I27" s="7">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="J26" s="1"/>
-    </row>
-    <row r="27" spans="1:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="81" t="s">
+      <c r="J27" s="1"/>
+    </row>
+    <row r="28" spans="1:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="54" t="s">
+        <v>32</v>
+      </c>
+      <c r="B28" s="55"/>
+      <c r="C28" s="55"/>
+      <c r="D28" s="55"/>
+      <c r="E28" s="23">
+        <f>SUM(E20:E27)</f>
+        <v>80</v>
+      </c>
+      <c r="F28" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="G28" s="18"/>
+      <c r="H28" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="I28" s="32">
+        <f>SUM(I20:I27)</f>
+        <v>450.6</v>
+      </c>
+      <c r="J28" s="2"/>
+    </row>
+    <row r="29" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="58" t="s">
+        <v>34</v>
+      </c>
+      <c r="B29" s="59"/>
+      <c r="C29" s="59"/>
+      <c r="D29" s="59"/>
+      <c r="E29" s="59"/>
+      <c r="F29" s="59"/>
+      <c r="G29" s="59"/>
+      <c r="H29" s="59"/>
+      <c r="I29" s="59"/>
+      <c r="J29" s="11"/>
+    </row>
+    <row r="30" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="28"/>
+      <c r="B30" s="28"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="28"/>
+      <c r="E30" s="28"/>
+      <c r="F30" s="28"/>
+      <c r="G30" s="28"/>
+      <c r="H30" s="28"/>
+      <c r="I30" s="28"/>
+      <c r="J30" s="11"/>
+    </row>
+    <row r="31" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="78" t="s">
+        <v>35</v>
+      </c>
+      <c r="B31" s="46"/>
+      <c r="C31" s="46"/>
+      <c r="D31" s="46"/>
+      <c r="E31" s="28"/>
+      <c r="F31" s="28"/>
+      <c r="G31" s="28"/>
+      <c r="H31" s="28"/>
+      <c r="I31" s="28"/>
+      <c r="J31" s="11"/>
+    </row>
+    <row r="32" spans="1:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="78" t="s">
+        <v>36</v>
+      </c>
+      <c r="B32" s="46"/>
+      <c r="C32" s="46"/>
+      <c r="D32" s="46"/>
+      <c r="E32" s="28"/>
+      <c r="F32" s="28"/>
+      <c r="G32" s="28"/>
+      <c r="H32" s="28"/>
+      <c r="I32" s="28"/>
+      <c r="J32" s="11"/>
+    </row>
+    <row r="33" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="79" t="s">
+        <v>13</v>
+      </c>
+      <c r="B33" s="80"/>
+      <c r="C33" s="80"/>
+      <c r="D33" s="80"/>
+      <c r="E33" s="28"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="28"/>
+      <c r="H33" s="28"/>
+      <c r="I33" s="28"/>
+      <c r="J33" s="11"/>
+    </row>
+    <row r="34" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="50" t="s">
+        <v>37</v>
+      </c>
+      <c r="B34" s="46"/>
+      <c r="C34" s="50">
+        <v>8116409</v>
+      </c>
+      <c r="D34" s="46"/>
+      <c r="E34" s="12"/>
+      <c r="F34" s="12"/>
+      <c r="G34" s="12"/>
+      <c r="H34" s="12"/>
+      <c r="I34" s="12"/>
+      <c r="J34" s="13"/>
+    </row>
+    <row r="35" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="50" t="s">
+        <v>38</v>
+      </c>
+      <c r="B35" s="46"/>
+      <c r="C35" s="88"/>
+      <c r="D35" s="46"/>
+      <c r="E35" s="12"/>
+      <c r="F35" s="12"/>
+      <c r="G35" s="12"/>
+      <c r="H35" s="12"/>
+      <c r="I35" s="12"/>
+      <c r="J35" s="13"/>
+    </row>
+    <row r="36" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="50" t="s">
         <v>39</v>
       </c>
-      <c r="B27" s="82"/>
-      <c r="C27" s="82"/>
-      <c r="D27" s="82"/>
-      <c r="E27" s="25">
-        <f>SUM(E19:E26)</f>
-        <v>80</v>
-      </c>
-      <c r="F27" s="18" t="s">
+      <c r="B36" s="46"/>
+      <c r="C36" s="78"/>
+      <c r="D36" s="46"/>
+      <c r="E36" s="12"/>
+      <c r="F36" s="12"/>
+      <c r="G36" s="12"/>
+      <c r="H36" s="12"/>
+      <c r="I36" s="12"/>
+      <c r="J36" s="13"/>
+    </row>
+    <row r="37" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="26"/>
+      <c r="B37" s="26"/>
+      <c r="C37" s="26"/>
+      <c r="D37" s="26"/>
+      <c r="E37" s="12"/>
+      <c r="F37" s="12"/>
+      <c r="G37" s="12"/>
+      <c r="H37" s="12"/>
+      <c r="I37" s="12"/>
+      <c r="J37" s="13"/>
+    </row>
+    <row r="38" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="26"/>
+      <c r="B38" s="26"/>
+      <c r="C38" s="26"/>
+      <c r="D38" s="26"/>
+      <c r="E38" s="12"/>
+      <c r="F38" s="12"/>
+      <c r="G38" s="12"/>
+      <c r="H38" s="12"/>
+      <c r="I38" s="12"/>
+      <c r="J38" s="13"/>
+    </row>
+    <row r="39" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="26"/>
+      <c r="B39" s="26"/>
+      <c r="C39" s="26"/>
+      <c r="D39" s="26"/>
+      <c r="E39" s="12"/>
+      <c r="F39" s="12"/>
+      <c r="G39" s="12"/>
+      <c r="H39" s="12"/>
+      <c r="I39" s="12"/>
+      <c r="J39" s="13"/>
+    </row>
+    <row r="40" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="26"/>
+      <c r="B40" s="26"/>
+      <c r="C40" s="26"/>
+      <c r="D40" s="26"/>
+      <c r="E40" s="12"/>
+      <c r="F40" s="12"/>
+      <c r="G40" s="12"/>
+      <c r="H40" s="12"/>
+      <c r="I40" s="12"/>
+      <c r="J40" s="13"/>
+    </row>
+    <row r="41" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="82" t="s">
         <v>40</v>
       </c>
-      <c r="G27" s="19"/>
-      <c r="H27" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="I27" s="35">
-        <f>SUM(I19:I26)</f>
-        <v>450.6</v>
-      </c>
-      <c r="J27" s="2"/>
-    </row>
-    <row r="28" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="87" t="s">
+      <c r="B41" s="46"/>
+      <c r="C41" s="46"/>
+      <c r="D41" s="46"/>
+      <c r="E41" s="46"/>
+      <c r="F41" s="46"/>
+      <c r="G41" s="46"/>
+      <c r="H41" s="46"/>
+      <c r="I41" s="46"/>
+      <c r="J41" s="13"/>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A42" s="81" t="s">
         <v>41</v>
       </c>
-      <c r="B28" s="88"/>
-      <c r="C28" s="88"/>
-      <c r="D28" s="88"/>
-      <c r="E28" s="88"/>
-      <c r="F28" s="88"/>
-      <c r="G28" s="88"/>
-      <c r="H28" s="88"/>
-      <c r="I28" s="88"/>
-      <c r="J28" s="12"/>
-    </row>
-    <row r="29" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="31"/>
-      <c r="B29" s="31"/>
-      <c r="C29" s="31"/>
-      <c r="D29" s="31"/>
-      <c r="E29" s="31"/>
-      <c r="F29" s="31"/>
-      <c r="G29" s="31"/>
-      <c r="H29" s="31"/>
-      <c r="I29" s="31"/>
-      <c r="J29" s="12"/>
-    </row>
-    <row r="30" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="74" t="s">
+      <c r="B42" s="46"/>
+      <c r="C42" s="46"/>
+      <c r="D42" s="46"/>
+      <c r="E42" s="46"/>
+      <c r="F42" s="67" t="s">
         <v>42</v>
       </c>
-      <c r="B30" s="48"/>
-      <c r="C30" s="48"/>
-      <c r="D30" s="48"/>
-      <c r="E30" s="31"/>
-      <c r="F30" s="31"/>
-      <c r="G30" s="31"/>
-      <c r="H30" s="31"/>
-      <c r="I30" s="31"/>
-      <c r="J30" s="12"/>
-    </row>
-    <row r="31" spans="1:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="74" t="s">
-        <v>43</v>
-      </c>
-      <c r="B31" s="48"/>
-      <c r="C31" s="48"/>
-      <c r="D31" s="48"/>
-      <c r="E31" s="31"/>
-      <c r="F31" s="31"/>
-      <c r="G31" s="31"/>
-      <c r="H31" s="31"/>
-      <c r="I31" s="31"/>
-      <c r="J31" s="12"/>
-    </row>
-    <row r="32" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="75" t="s">
-        <v>19</v>
-      </c>
-      <c r="B32" s="76"/>
-      <c r="C32" s="76"/>
-      <c r="D32" s="76"/>
-      <c r="E32" s="31"/>
-      <c r="F32" s="31"/>
-      <c r="G32" s="31"/>
-      <c r="H32" s="31"/>
-      <c r="I32" s="31"/>
-      <c r="J32" s="12"/>
-    </row>
-    <row r="33" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="49" t="s">
-        <v>44</v>
-      </c>
-      <c r="B33" s="48"/>
-      <c r="C33" s="49">
-        <v>8116409</v>
-      </c>
-      <c r="D33" s="48"/>
-      <c r="E33" s="13"/>
-      <c r="F33" s="13"/>
-      <c r="G33" s="13"/>
-      <c r="H33" s="13"/>
-      <c r="I33" s="13"/>
-      <c r="J33" s="14"/>
-    </row>
-    <row r="34" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="49" t="s">
-        <v>45</v>
-      </c>
-      <c r="B34" s="48"/>
-      <c r="C34" s="63"/>
-      <c r="D34" s="48"/>
-      <c r="E34" s="13"/>
-      <c r="F34" s="13"/>
-      <c r="G34" s="13"/>
-      <c r="H34" s="13"/>
-      <c r="I34" s="13"/>
-      <c r="J34" s="14"/>
-    </row>
-    <row r="35" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="49" t="s">
-        <v>46</v>
-      </c>
-      <c r="B35" s="48"/>
-      <c r="C35" s="74"/>
-      <c r="D35" s="48"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="13"/>
-      <c r="G35" s="13"/>
-      <c r="H35" s="13"/>
-      <c r="I35" s="13"/>
-      <c r="J35" s="14"/>
-    </row>
-    <row r="36" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="28"/>
-      <c r="B36" s="28"/>
-      <c r="C36" s="28"/>
-      <c r="D36" s="28"/>
-      <c r="E36" s="13"/>
-      <c r="F36" s="13"/>
-      <c r="G36" s="13"/>
-      <c r="H36" s="13"/>
-      <c r="I36" s="13"/>
-      <c r="J36" s="14"/>
-    </row>
-    <row r="37" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="28"/>
-      <c r="B37" s="28"/>
-      <c r="C37" s="28"/>
-      <c r="D37" s="28"/>
-      <c r="E37" s="13"/>
-      <c r="F37" s="13"/>
-      <c r="G37" s="13"/>
-      <c r="H37" s="13"/>
-      <c r="I37" s="13"/>
-      <c r="J37" s="14"/>
-    </row>
-    <row r="38" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="28"/>
-      <c r="B38" s="28"/>
-      <c r="C38" s="28"/>
-      <c r="D38" s="28"/>
-      <c r="E38" s="13"/>
-      <c r="F38" s="13"/>
-      <c r="G38" s="13"/>
-      <c r="H38" s="13"/>
-      <c r="I38" s="13"/>
-      <c r="J38" s="14"/>
-    </row>
-    <row r="39" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="28"/>
-      <c r="B39" s="28"/>
-      <c r="C39" s="28"/>
-      <c r="D39" s="28"/>
-      <c r="E39" s="13"/>
-      <c r="F39" s="13"/>
-      <c r="G39" s="13"/>
-      <c r="H39" s="13"/>
-      <c r="I39" s="13"/>
-      <c r="J39" s="14"/>
-    </row>
-    <row r="40" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="47" t="s">
-        <v>47</v>
-      </c>
-      <c r="B40" s="48"/>
-      <c r="C40" s="48"/>
-      <c r="D40" s="48"/>
-      <c r="E40" s="48"/>
-      <c r="F40" s="48"/>
-      <c r="G40" s="48"/>
-      <c r="H40" s="48"/>
-      <c r="I40" s="48"/>
-      <c r="J40" s="14"/>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A41" s="77" t="s">
-        <v>48</v>
-      </c>
-      <c r="B41" s="48"/>
-      <c r="C41" s="48"/>
-      <c r="D41" s="48"/>
-      <c r="E41" s="48"/>
-      <c r="F41" s="66" t="s">
-        <v>49</v>
-      </c>
-      <c r="G41" s="48"/>
-      <c r="H41" s="48"/>
-      <c r="I41" s="48"/>
-      <c r="J41" s="15"/>
+      <c r="G42" s="46"/>
+      <c r="H42" s="46"/>
+      <c r="I42" s="46"/>
+      <c r="J42" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="45">
+    <mergeCell ref="A41:I41"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="F7:I11"/>
+    <mergeCell ref="I12:I15"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="H12:H15"/>
+    <mergeCell ref="F12:G13"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A5:E7"/>
+    <mergeCell ref="F42:I42"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A25:D25"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F15:G15"/>
     <mergeCell ref="E2:H2"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A29:I29"/>
     <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="F6:I6"/>
     <mergeCell ref="A9:E9"/>
-    <mergeCell ref="A7:E7"/>
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A28:I28"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="F6:I6"/>
-    <mergeCell ref="F41:I41"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="B14:E14"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A41:E41"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A40:I40"/>
-    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A10:E10"/>
     <mergeCell ref="A11:E11"/>
-    <mergeCell ref="F7:I10"/>
-    <mergeCell ref="I11:I14"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="H11:H14"/>
-    <mergeCell ref="F11:G12"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="A20:D20"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="F41" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="F42" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
-  <pageMargins left="0.59055118110236227" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageMargins left="0.39370078740157483" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
   <drawing r:id="rId3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Customer PO column to CI/PL templates (E20+)
Both templates now show per-item Customer PO in column E so consolidated
invoices with mixed POs remain traceable. G16 (PO No) and shipping mark
PO cells join unique POs with commas.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/commercial_invoice.xlsx
+++ b/templates/commercial_invoice.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rotork-my.sharepoint.com/personal/jeongtaek_bang_rotork_com/Documents/바탕 화면/업무/NOAH ACTUATION/noahAutomation/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="84" documentId="11_482B29FEF0C7F80AEE82E0F7E4E761DFCF1F255D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{642D3CBD-35D9-4568-811B-D2C4B4C6954C}"/>
+  <xr:revisionPtr revIDLastSave="107" documentId="11_482B29FEF0C7F80AEE82E0F7E4E761DFCF1F255D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94D4BCAE-56E9-4AC8-B7A0-7A7C39509C3C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="48">
   <si>
     <t>Commercial Invoice</t>
   </si>
@@ -189,6 +189,10 @@
   </si>
   <si>
     <t xml:space="preserve">HS CODE: </t>
+    <phoneticPr fontId="17" type="noConversion"/>
+  </si>
+  <si>
+    <t>PO No.</t>
     <phoneticPr fontId="17" type="noConversion"/>
   </si>
 </sst>
@@ -530,7 +534,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -558,9 +562,6 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" indent="3" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -585,9 +586,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -650,9 +648,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -790,6 +785,9 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -870,7 +868,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>783796</xdr:colOff>
+      <xdr:colOff>658467</xdr:colOff>
       <xdr:row>37</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -1204,28 +1202,28 @@
   <dimension ref="A1:J42"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.5" style="41" customWidth="1"/>
-    <col min="2" max="2" width="5.6640625" style="41" customWidth="1"/>
-    <col min="3" max="3" width="13.83203125" style="41" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.33203125" style="41" customWidth="1"/>
-    <col min="5" max="5" width="9.5" style="41" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" style="41" customWidth="1"/>
-    <col min="7" max="7" width="11.6640625" style="41" customWidth="1"/>
-    <col min="8" max="8" width="11.1640625" style="41" customWidth="1"/>
-    <col min="9" max="9" width="24.5" style="41" customWidth="1"/>
-    <col min="10" max="10" width="14" style="41" customWidth="1"/>
+    <col min="1" max="1" width="10.5" style="38" customWidth="1"/>
+    <col min="2" max="2" width="5.6640625" style="38" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" style="38" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.33203125" style="38" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" style="38" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" style="38" customWidth="1"/>
+    <col min="7" max="7" width="13.83203125" style="38" customWidth="1"/>
+    <col min="8" max="8" width="11.1640625" style="38" customWidth="1"/>
+    <col min="9" max="9" width="21.83203125" style="38" customWidth="1"/>
+    <col min="10" max="10" width="14" style="38" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="45"/>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
+      <c r="A1" s="42"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1233,12 +1231,12 @@
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
-      <c r="E2" s="49" t="s">
+      <c r="E2" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
     </row>
@@ -1255,646 +1253,646 @@
       <c r="J3" s="2"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="51" t="s">
+      <c r="A4" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="52"/>
-      <c r="C4" s="52"/>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
-      <c r="F4" s="30" t="s">
+      <c r="B4" s="49"/>
+      <c r="C4" s="49"/>
+      <c r="D4" s="49"/>
+      <c r="E4" s="50"/>
+      <c r="F4" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="G4" s="29"/>
-      <c r="H4" s="19" t="s">
+      <c r="G4" s="27"/>
+      <c r="H4" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="29"/>
+      <c r="I4" s="27"/>
       <c r="J4" s="1"/>
     </row>
     <row r="5" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="61" t="s">
+      <c r="A5" s="58" t="s">
         <v>45</v>
       </c>
-      <c r="B5" s="90"/>
-      <c r="C5" s="90"/>
-      <c r="D5" s="90"/>
-      <c r="E5" s="91"/>
-      <c r="F5" s="44" t="s">
+      <c r="B5" s="87"/>
+      <c r="C5" s="87"/>
+      <c r="D5" s="87"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="41" t="s">
         <v>44</v>
       </c>
-      <c r="G5" s="25"/>
-      <c r="H5" s="21" t="s">
+      <c r="G5" s="23"/>
+      <c r="H5" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="I5" s="25"/>
+      <c r="I5" s="23"/>
       <c r="J5" s="1"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="92"/>
-      <c r="B6" s="90"/>
-      <c r="C6" s="90"/>
-      <c r="D6" s="90"/>
-      <c r="E6" s="91"/>
-      <c r="F6" s="60" t="s">
+      <c r="A6" s="89"/>
+      <c r="B6" s="87"/>
+      <c r="C6" s="87"/>
+      <c r="D6" s="87"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="57" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="52"/>
-      <c r="H6" s="52"/>
-      <c r="I6" s="53"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="49"/>
+      <c r="I6" s="50"/>
       <c r="J6" s="1"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="93"/>
-      <c r="B7" s="94"/>
-      <c r="C7" s="94"/>
-      <c r="D7" s="94"/>
-      <c r="E7" s="95"/>
-      <c r="F7" s="83"/>
-      <c r="G7" s="46"/>
-      <c r="H7" s="46"/>
-      <c r="I7" s="75"/>
+      <c r="A7" s="90"/>
+      <c r="B7" s="91"/>
+      <c r="C7" s="91"/>
+      <c r="D7" s="91"/>
+      <c r="E7" s="92"/>
+      <c r="F7" s="80"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="43"/>
+      <c r="I7" s="72"/>
       <c r="J7" s="1"/>
     </row>
     <row r="8" spans="1:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="51" t="s">
+      <c r="A8" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="52"/>
-      <c r="C8" s="52"/>
-      <c r="D8" s="52"/>
-      <c r="E8" s="53"/>
-      <c r="F8" s="84"/>
-      <c r="G8" s="46"/>
-      <c r="H8" s="46"/>
-      <c r="I8" s="75"/>
+      <c r="B8" s="49"/>
+      <c r="C8" s="49"/>
+      <c r="D8" s="49"/>
+      <c r="E8" s="50"/>
+      <c r="F8" s="81"/>
+      <c r="G8" s="43"/>
+      <c r="H8" s="43"/>
+      <c r="I8" s="72"/>
       <c r="J8" s="1"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="61"/>
-      <c r="B9" s="62"/>
-      <c r="C9" s="62"/>
-      <c r="D9" s="62"/>
-      <c r="E9" s="63"/>
-      <c r="F9" s="84"/>
-      <c r="G9" s="46"/>
-      <c r="H9" s="46"/>
-      <c r="I9" s="75"/>
+      <c r="A9" s="58"/>
+      <c r="B9" s="59"/>
+      <c r="C9" s="59"/>
+      <c r="D9" s="59"/>
+      <c r="E9" s="60"/>
+      <c r="F9" s="81"/>
+      <c r="G9" s="43"/>
+      <c r="H9" s="43"/>
+      <c r="I9" s="72"/>
       <c r="J9" s="4"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="61"/>
-      <c r="B10" s="62"/>
-      <c r="C10" s="62"/>
-      <c r="D10" s="62"/>
-      <c r="E10" s="63"/>
-      <c r="F10" s="84"/>
-      <c r="G10" s="46"/>
-      <c r="H10" s="46"/>
-      <c r="I10" s="75"/>
+      <c r="A10" s="58"/>
+      <c r="B10" s="59"/>
+      <c r="C10" s="59"/>
+      <c r="D10" s="59"/>
+      <c r="E10" s="60"/>
+      <c r="F10" s="81"/>
+      <c r="G10" s="43"/>
+      <c r="H10" s="43"/>
+      <c r="I10" s="72"/>
       <c r="J10" s="4"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="64"/>
-      <c r="B11" s="65"/>
-      <c r="C11" s="65"/>
-      <c r="D11" s="65"/>
-      <c r="E11" s="66"/>
-      <c r="F11" s="85"/>
-      <c r="G11" s="57"/>
-      <c r="H11" s="57"/>
-      <c r="I11" s="48"/>
+      <c r="A11" s="61"/>
+      <c r="B11" s="62"/>
+      <c r="C11" s="62"/>
+      <c r="D11" s="62"/>
+      <c r="E11" s="63"/>
+      <c r="F11" s="82"/>
+      <c r="G11" s="54"/>
+      <c r="H11" s="54"/>
+      <c r="I11" s="45"/>
       <c r="J11" s="2"/>
     </row>
     <row r="12" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="51" t="s">
+      <c r="A12" s="48" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="52"/>
-      <c r="C12" s="52"/>
-      <c r="D12" s="52"/>
-      <c r="E12" s="53"/>
-      <c r="F12" s="60" t="s">
+      <c r="B12" s="49"/>
+      <c r="C12" s="49"/>
+      <c r="D12" s="49"/>
+      <c r="E12" s="50"/>
+      <c r="F12" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="G12" s="53"/>
-      <c r="H12" s="87" t="s">
+      <c r="G12" s="50"/>
+      <c r="H12" s="84" t="s">
         <v>46</v>
       </c>
-      <c r="I12" s="86" t="s">
+      <c r="I12" s="83" t="s">
         <v>8</v>
       </c>
       <c r="J12" s="2"/>
     </row>
     <row r="13" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="56"/>
-      <c r="B13" s="57"/>
-      <c r="C13" s="57"/>
-      <c r="D13" s="57"/>
-      <c r="E13" s="48"/>
-      <c r="F13" s="84"/>
-      <c r="G13" s="75"/>
-      <c r="H13" s="46"/>
-      <c r="I13" s="75"/>
+      <c r="A13" s="53"/>
+      <c r="B13" s="54"/>
+      <c r="C13" s="54"/>
+      <c r="D13" s="54"/>
+      <c r="E13" s="45"/>
+      <c r="F13" s="81"/>
+      <c r="G13" s="72"/>
+      <c r="H13" s="43"/>
+      <c r="I13" s="72"/>
       <c r="J13" s="2"/>
     </row>
     <row r="14" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="31" t="s">
+      <c r="A14" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="70" t="s">
+      <c r="B14" s="67" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="71"/>
-      <c r="D14" s="71"/>
-      <c r="E14" s="69"/>
-      <c r="F14" s="74" t="s">
+      <c r="C14" s="68"/>
+      <c r="D14" s="68"/>
+      <c r="E14" s="66"/>
+      <c r="F14" s="71" t="s">
         <v>11</v>
       </c>
-      <c r="G14" s="75"/>
-      <c r="H14" s="46"/>
-      <c r="I14" s="75"/>
+      <c r="G14" s="72"/>
+      <c r="H14" s="43"/>
+      <c r="I14" s="72"/>
       <c r="J14" s="2"/>
     </row>
     <row r="15" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="31" t="s">
+      <c r="A15" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="70"/>
-      <c r="C15" s="71"/>
-      <c r="D15" s="71"/>
-      <c r="E15" s="69"/>
-      <c r="F15" s="47" t="s">
+      <c r="B15" s="67"/>
+      <c r="C15" s="68"/>
+      <c r="D15" s="68"/>
+      <c r="E15" s="66"/>
+      <c r="F15" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="G15" s="48"/>
-      <c r="H15" s="57"/>
-      <c r="I15" s="48"/>
+      <c r="G15" s="45"/>
+      <c r="H15" s="54"/>
+      <c r="I15" s="45"/>
       <c r="J15" s="2"/>
     </row>
     <row r="16" spans="1:10" ht="17.850000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="76" t="s">
+      <c r="A16" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="71"/>
-      <c r="C16" s="71"/>
-      <c r="D16" s="68">
-        <v>46030</v>
-      </c>
-      <c r="E16" s="69"/>
-      <c r="F16" s="24" t="s">
+      <c r="B16" s="68"/>
+      <c r="C16" s="68"/>
+      <c r="D16" s="65"/>
+      <c r="E16" s="66"/>
+      <c r="F16" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="G16" s="20"/>
-      <c r="H16" s="22" t="s">
+      <c r="G16" s="18"/>
+      <c r="H16" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="I16" s="27"/>
+      <c r="I16" s="25"/>
       <c r="J16" s="1"/>
     </row>
     <row r="17" spans="1:10" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="33"/>
-      <c r="B17" s="33"/>
-      <c r="C17" s="33"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="34"/>
-      <c r="F17" s="35"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="36"/>
-      <c r="I17" s="37"/>
+      <c r="A17" s="31"/>
+      <c r="B17" s="31"/>
+      <c r="C17" s="31"/>
+      <c r="D17" s="36"/>
+      <c r="E17" s="32"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="34"/>
+      <c r="I17" s="35"/>
       <c r="J17" s="1"/>
     </row>
     <row r="18" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="89" t="s">
+      <c r="A18" s="86" t="s">
         <v>18</v>
       </c>
-      <c r="B18" s="71"/>
-      <c r="C18" s="71"/>
-      <c r="D18" s="71"/>
-      <c r="E18" s="39" t="s">
+      <c r="B18" s="68"/>
+      <c r="C18" s="68"/>
+      <c r="D18" s="68"/>
+      <c r="E18" s="93" t="s">
+        <v>47</v>
+      </c>
+      <c r="F18" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="F18" s="40"/>
-      <c r="G18" s="39" t="s">
+      <c r="G18" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="H18" s="39" t="s">
+      <c r="H18" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="I18" s="39"/>
-      <c r="J18" s="11"/>
+      <c r="I18" s="37"/>
+      <c r="J18" s="10"/>
     </row>
     <row r="19" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="77" t="s">
+      <c r="A19" s="74" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="52"/>
-      <c r="C19" s="52"/>
-      <c r="D19" s="52"/>
+      <c r="B19" s="49"/>
+      <c r="C19" s="49"/>
+      <c r="D19" s="49"/>
       <c r="E19" s="5"/>
-      <c r="F19" s="3"/>
+      <c r="F19" s="5"/>
       <c r="G19" s="3"/>
-      <c r="H19" s="16"/>
-      <c r="I19" s="16"/>
+      <c r="H19" s="15"/>
+      <c r="I19" s="15"/>
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="73" t="s">
+      <c r="A20" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="46"/>
-      <c r="C20" s="46"/>
-      <c r="D20" s="46"/>
-      <c r="E20" s="6">
+      <c r="B20" s="43"/>
+      <c r="C20" s="43"/>
+      <c r="D20" s="43"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6">
         <v>10</v>
       </c>
-      <c r="F20" s="1"/>
-      <c r="G20" s="42">
+      <c r="G20" s="39">
         <v>24</v>
       </c>
-      <c r="H20" s="10" t="s">
+      <c r="H20" s="9" t="s">
         <v>24</v>
       </c>
       <c r="I20" s="7">
         <f t="shared" ref="I20:I27" si="0">E20*G20</f>
-        <v>240</v>
+        <v>0</v>
       </c>
       <c r="J20" s="1"/>
     </row>
     <row r="21" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="73" t="s">
+      <c r="A21" s="70" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="46"/>
-      <c r="C21" s="46"/>
-      <c r="D21" s="46"/>
-      <c r="E21" s="6">
+      <c r="B21" s="43"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6">
         <v>10</v>
       </c>
-      <c r="F21" s="1"/>
-      <c r="G21" s="42">
+      <c r="G21" s="39">
         <v>1.26</v>
       </c>
-      <c r="H21" s="10" t="s">
+      <c r="H21" s="9" t="s">
         <v>24</v>
       </c>
       <c r="I21" s="7">
         <f t="shared" si="0"/>
-        <v>12.6</v>
+        <v>0</v>
       </c>
       <c r="J21" s="1"/>
     </row>
     <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="73" t="s">
+      <c r="A22" s="70" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="46"/>
-      <c r="C22" s="46"/>
-      <c r="D22" s="46"/>
-      <c r="E22" s="6">
+      <c r="B22" s="43"/>
+      <c r="C22" s="43"/>
+      <c r="D22" s="43"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6">
         <v>10</v>
       </c>
-      <c r="F22" s="1"/>
-      <c r="G22" s="42">
+      <c r="G22" s="39">
         <v>3.7</v>
       </c>
-      <c r="H22" s="10" t="s">
+      <c r="H22" s="9" t="s">
         <v>24</v>
       </c>
       <c r="I22" s="7">
         <f t="shared" si="0"/>
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="J22" s="1"/>
     </row>
     <row r="23" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="73" t="s">
+      <c r="A23" s="70" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="46"/>
-      <c r="C23" s="46"/>
-      <c r="D23" s="46"/>
-      <c r="E23" s="6">
+      <c r="B23" s="43"/>
+      <c r="C23" s="43"/>
+      <c r="D23" s="43"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6">
         <v>10</v>
       </c>
-      <c r="F23" s="1"/>
-      <c r="G23" s="42">
+      <c r="G23" s="39">
         <v>3.9</v>
       </c>
-      <c r="H23" s="10" t="s">
+      <c r="H23" s="9" t="s">
         <v>24</v>
       </c>
       <c r="I23" s="7">
         <f t="shared" si="0"/>
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="J23" s="1"/>
     </row>
     <row r="24" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="73" t="s">
+      <c r="A24" s="70" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="46"/>
-      <c r="C24" s="46"/>
-      <c r="D24" s="46"/>
-      <c r="E24" s="6">
+      <c r="B24" s="43"/>
+      <c r="C24" s="43"/>
+      <c r="D24" s="43"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6">
         <v>10</v>
       </c>
-      <c r="F24" s="1"/>
-      <c r="G24" s="42">
+      <c r="G24" s="39">
         <v>3.9</v>
       </c>
-      <c r="H24" s="10" t="s">
+      <c r="H24" s="9" t="s">
         <v>24</v>
       </c>
       <c r="I24" s="7">
         <f t="shared" si="0"/>
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="J24" s="1"/>
     </row>
     <row r="25" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="73" t="s">
+      <c r="A25" s="70" t="s">
         <v>29</v>
       </c>
-      <c r="B25" s="46"/>
-      <c r="C25" s="46"/>
-      <c r="D25" s="46"/>
-      <c r="E25" s="6">
+      <c r="B25" s="43"/>
+      <c r="C25" s="43"/>
+      <c r="D25" s="43"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6">
         <v>10</v>
       </c>
-      <c r="F25" s="1"/>
-      <c r="G25" s="42">
+      <c r="G25" s="39">
         <v>2.5</v>
       </c>
-      <c r="H25" s="10" t="s">
+      <c r="H25" s="9" t="s">
         <v>24</v>
       </c>
       <c r="I25" s="7">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="J25" s="1"/>
     </row>
     <row r="26" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="73" t="s">
+      <c r="A26" s="70" t="s">
         <v>30</v>
       </c>
-      <c r="B26" s="46"/>
-      <c r="C26" s="46"/>
-      <c r="D26" s="46"/>
-      <c r="E26" s="6">
+      <c r="B26" s="43"/>
+      <c r="C26" s="43"/>
+      <c r="D26" s="43"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6">
         <v>10</v>
       </c>
-      <c r="F26" s="1"/>
-      <c r="G26" s="42">
+      <c r="G26" s="39">
         <v>2.9</v>
       </c>
-      <c r="H26" s="10" t="s">
+      <c r="H26" s="9" t="s">
         <v>24</v>
       </c>
       <c r="I26" s="7">
         <f t="shared" si="0"/>
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="J26" s="1"/>
     </row>
     <row r="27" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="72" t="s">
+      <c r="A27" s="69" t="s">
         <v>31</v>
       </c>
-      <c r="B27" s="57"/>
-      <c r="C27" s="57"/>
-      <c r="D27" s="57"/>
-      <c r="E27" s="8">
+      <c r="B27" s="54"/>
+      <c r="C27" s="54"/>
+      <c r="D27" s="54"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8">
         <v>10</v>
       </c>
-      <c r="F27" s="9"/>
-      <c r="G27" s="43">
+      <c r="G27" s="40">
         <v>2.9</v>
       </c>
-      <c r="H27" s="15" t="s">
+      <c r="H27" s="14" t="s">
         <v>24</v>
       </c>
       <c r="I27" s="7">
         <f t="shared" si="0"/>
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="J27" s="1"/>
     </row>
     <row r="28" spans="1:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="54" t="s">
+      <c r="A28" s="51" t="s">
         <v>32</v>
       </c>
-      <c r="B28" s="55"/>
-      <c r="C28" s="55"/>
-      <c r="D28" s="55"/>
-      <c r="E28" s="23">
-        <f>SUM(E20:E27)</f>
+      <c r="B28" s="52"/>
+      <c r="C28" s="52"/>
+      <c r="D28" s="52"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="21">
+        <f>SUM(F20:F27)</f>
         <v>80</v>
       </c>
-      <c r="F28" s="17" t="s">
+      <c r="G28" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="G28" s="18"/>
-      <c r="H28" s="17" t="s">
+      <c r="H28" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="I28" s="32">
+      <c r="I28" s="30">
         <f>SUM(I20:I27)</f>
-        <v>450.6</v>
+        <v>0</v>
       </c>
       <c r="J28" s="2"/>
     </row>
     <row r="29" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="58" t="s">
+      <c r="A29" s="55" t="s">
         <v>34</v>
       </c>
-      <c r="B29" s="59"/>
-      <c r="C29" s="59"/>
-      <c r="D29" s="59"/>
-      <c r="E29" s="59"/>
-      <c r="F29" s="59"/>
-      <c r="G29" s="59"/>
-      <c r="H29" s="59"/>
-      <c r="I29" s="59"/>
-      <c r="J29" s="11"/>
+      <c r="B29" s="56"/>
+      <c r="C29" s="56"/>
+      <c r="D29" s="56"/>
+      <c r="E29" s="56"/>
+      <c r="F29" s="56"/>
+      <c r="G29" s="56"/>
+      <c r="H29" s="56"/>
+      <c r="I29" s="56"/>
+      <c r="J29" s="10"/>
     </row>
     <row r="30" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="28"/>
-      <c r="B30" s="28"/>
-      <c r="C30" s="28"/>
-      <c r="D30" s="28"/>
-      <c r="E30" s="28"/>
-      <c r="F30" s="28"/>
-      <c r="G30" s="28"/>
-      <c r="H30" s="28"/>
-      <c r="I30" s="28"/>
-      <c r="J30" s="11"/>
+      <c r="A30" s="26"/>
+      <c r="B30" s="26"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="26"/>
+      <c r="G30" s="26"/>
+      <c r="H30" s="26"/>
+      <c r="I30" s="26"/>
+      <c r="J30" s="10"/>
     </row>
     <row r="31" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="78" t="s">
+      <c r="A31" s="75" t="s">
         <v>35</v>
       </c>
-      <c r="B31" s="46"/>
-      <c r="C31" s="46"/>
-      <c r="D31" s="46"/>
-      <c r="E31" s="28"/>
-      <c r="F31" s="28"/>
-      <c r="G31" s="28"/>
-      <c r="H31" s="28"/>
-      <c r="I31" s="28"/>
-      <c r="J31" s="11"/>
+      <c r="B31" s="43"/>
+      <c r="C31" s="43"/>
+      <c r="D31" s="43"/>
+      <c r="E31" s="26"/>
+      <c r="F31" s="26"/>
+      <c r="G31" s="26"/>
+      <c r="H31" s="26"/>
+      <c r="I31" s="26"/>
+      <c r="J31" s="10"/>
     </row>
     <row r="32" spans="1:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="78" t="s">
+      <c r="A32" s="75" t="s">
         <v>36</v>
       </c>
-      <c r="B32" s="46"/>
-      <c r="C32" s="46"/>
-      <c r="D32" s="46"/>
-      <c r="E32" s="28"/>
-      <c r="F32" s="28"/>
-      <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
-      <c r="I32" s="28"/>
-      <c r="J32" s="11"/>
+      <c r="B32" s="43"/>
+      <c r="C32" s="43"/>
+      <c r="D32" s="43"/>
+      <c r="E32" s="26"/>
+      <c r="F32" s="26"/>
+      <c r="G32" s="26"/>
+      <c r="H32" s="26"/>
+      <c r="I32" s="26"/>
+      <c r="J32" s="10"/>
     </row>
     <row r="33" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="79" t="s">
+      <c r="A33" s="76" t="s">
         <v>13</v>
       </c>
-      <c r="B33" s="80"/>
-      <c r="C33" s="80"/>
-      <c r="D33" s="80"/>
-      <c r="E33" s="28"/>
-      <c r="F33" s="28"/>
-      <c r="G33" s="28"/>
-      <c r="H33" s="28"/>
-      <c r="I33" s="28"/>
-      <c r="J33" s="11"/>
+      <c r="B33" s="77"/>
+      <c r="C33" s="77"/>
+      <c r="D33" s="77"/>
+      <c r="E33" s="26"/>
+      <c r="F33" s="26"/>
+      <c r="G33" s="26"/>
+      <c r="H33" s="26"/>
+      <c r="I33" s="26"/>
+      <c r="J33" s="10"/>
     </row>
     <row r="34" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="50" t="s">
+      <c r="A34" s="47" t="s">
         <v>37</v>
       </c>
-      <c r="B34" s="46"/>
-      <c r="C34" s="50">
+      <c r="B34" s="43"/>
+      <c r="C34" s="47">
         <v>8116409</v>
       </c>
-      <c r="D34" s="46"/>
-      <c r="E34" s="12"/>
-      <c r="F34" s="12"/>
-      <c r="G34" s="12"/>
-      <c r="H34" s="12"/>
-      <c r="I34" s="12"/>
-      <c r="J34" s="13"/>
+      <c r="D34" s="43"/>
+      <c r="E34" s="11"/>
+      <c r="F34" s="11"/>
+      <c r="G34" s="11"/>
+      <c r="H34" s="11"/>
+      <c r="I34" s="11"/>
+      <c r="J34" s="12"/>
     </row>
     <row r="35" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="50" t="s">
+      <c r="A35" s="47" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="46"/>
-      <c r="C35" s="88"/>
-      <c r="D35" s="46"/>
-      <c r="E35" s="12"/>
-      <c r="F35" s="12"/>
-      <c r="G35" s="12"/>
-      <c r="H35" s="12"/>
-      <c r="I35" s="12"/>
-      <c r="J35" s="13"/>
+      <c r="B35" s="43"/>
+      <c r="C35" s="85"/>
+      <c r="D35" s="43"/>
+      <c r="E35" s="11"/>
+      <c r="F35" s="11"/>
+      <c r="G35" s="11"/>
+      <c r="H35" s="11"/>
+      <c r="I35" s="11"/>
+      <c r="J35" s="12"/>
     </row>
     <row r="36" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="50" t="s">
+      <c r="A36" s="47" t="s">
         <v>39</v>
       </c>
-      <c r="B36" s="46"/>
-      <c r="C36" s="78"/>
-      <c r="D36" s="46"/>
-      <c r="E36" s="12"/>
-      <c r="F36" s="12"/>
-      <c r="G36" s="12"/>
-      <c r="H36" s="12"/>
-      <c r="I36" s="12"/>
-      <c r="J36" s="13"/>
+      <c r="B36" s="43"/>
+      <c r="C36" s="75"/>
+      <c r="D36" s="43"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="11"/>
+      <c r="G36" s="11"/>
+      <c r="H36" s="11"/>
+      <c r="I36" s="11"/>
+      <c r="J36" s="12"/>
     </row>
     <row r="37" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="26"/>
-      <c r="B37" s="26"/>
-      <c r="C37" s="26"/>
-      <c r="D37" s="26"/>
-      <c r="E37" s="12"/>
-      <c r="F37" s="12"/>
-      <c r="G37" s="12"/>
-      <c r="H37" s="12"/>
-      <c r="I37" s="12"/>
-      <c r="J37" s="13"/>
+      <c r="A37" s="24"/>
+      <c r="B37" s="24"/>
+      <c r="C37" s="24"/>
+      <c r="D37" s="24"/>
+      <c r="E37" s="11"/>
+      <c r="F37" s="11"/>
+      <c r="G37" s="11"/>
+      <c r="H37" s="11"/>
+      <c r="I37" s="11"/>
+      <c r="J37" s="12"/>
     </row>
     <row r="38" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="26"/>
-      <c r="B38" s="26"/>
-      <c r="C38" s="26"/>
-      <c r="D38" s="26"/>
-      <c r="E38" s="12"/>
-      <c r="F38" s="12"/>
-      <c r="G38" s="12"/>
-      <c r="H38" s="12"/>
-      <c r="I38" s="12"/>
-      <c r="J38" s="13"/>
+      <c r="A38" s="24"/>
+      <c r="B38" s="24"/>
+      <c r="C38" s="24"/>
+      <c r="D38" s="24"/>
+      <c r="E38" s="11"/>
+      <c r="F38" s="11"/>
+      <c r="G38" s="11"/>
+      <c r="H38" s="11"/>
+      <c r="I38" s="11"/>
+      <c r="J38" s="12"/>
     </row>
     <row r="39" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="26"/>
-      <c r="B39" s="26"/>
-      <c r="C39" s="26"/>
-      <c r="D39" s="26"/>
-      <c r="E39" s="12"/>
-      <c r="F39" s="12"/>
-      <c r="G39" s="12"/>
-      <c r="H39" s="12"/>
-      <c r="I39" s="12"/>
-      <c r="J39" s="13"/>
+      <c r="A39" s="24"/>
+      <c r="B39" s="24"/>
+      <c r="C39" s="24"/>
+      <c r="D39" s="24"/>
+      <c r="E39" s="11"/>
+      <c r="F39" s="11"/>
+      <c r="G39" s="11"/>
+      <c r="H39" s="11"/>
+      <c r="I39" s="11"/>
+      <c r="J39" s="12"/>
     </row>
     <row r="40" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="26"/>
-      <c r="B40" s="26"/>
-      <c r="C40" s="26"/>
-      <c r="D40" s="26"/>
-      <c r="E40" s="12"/>
-      <c r="F40" s="12"/>
-      <c r="G40" s="12"/>
-      <c r="H40" s="12"/>
-      <c r="I40" s="12"/>
-      <c r="J40" s="13"/>
+      <c r="A40" s="24"/>
+      <c r="B40" s="24"/>
+      <c r="C40" s="24"/>
+      <c r="D40" s="24"/>
+      <c r="E40" s="11"/>
+      <c r="F40" s="11"/>
+      <c r="G40" s="11"/>
+      <c r="H40" s="11"/>
+      <c r="I40" s="11"/>
+      <c r="J40" s="12"/>
     </row>
     <row r="41" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="82" t="s">
+      <c r="A41" s="79" t="s">
         <v>40</v>
       </c>
-      <c r="B41" s="46"/>
-      <c r="C41" s="46"/>
-      <c r="D41" s="46"/>
-      <c r="E41" s="46"/>
-      <c r="F41" s="46"/>
-      <c r="G41" s="46"/>
-      <c r="H41" s="46"/>
-      <c r="I41" s="46"/>
-      <c r="J41" s="13"/>
+      <c r="B41" s="43"/>
+      <c r="C41" s="43"/>
+      <c r="D41" s="43"/>
+      <c r="E41" s="43"/>
+      <c r="F41" s="43"/>
+      <c r="G41" s="43"/>
+      <c r="H41" s="43"/>
+      <c r="I41" s="43"/>
+      <c r="J41" s="12"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A42" s="81" t="s">
+      <c r="A42" s="78" t="s">
         <v>41</v>
       </c>
-      <c r="B42" s="46"/>
-      <c r="C42" s="46"/>
-      <c r="D42" s="46"/>
-      <c r="E42" s="46"/>
-      <c r="F42" s="67" t="s">
+      <c r="B42" s="43"/>
+      <c r="C42" s="43"/>
+      <c r="D42" s="43"/>
+      <c r="E42" s="43"/>
+      <c r="F42" s="64" t="s">
         <v>42</v>
       </c>
-      <c r="G42" s="46"/>
-      <c r="H42" s="46"/>
-      <c r="I42" s="46"/>
-      <c r="J42" s="14"/>
+      <c r="G42" s="43"/>
+      <c r="H42" s="43"/>
+      <c r="I42" s="43"/>
+      <c r="J42" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="45">
@@ -1950,6 +1948,9 @@
   </hyperlinks>
   <pageMargins left="0.39370078740157483" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <headerFooter>
+    <oddFooter>Page &amp;P of &amp;N</oddFooter>
+  </headerFooter>
   <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
템플릿 — HS 코드 8481.90.3000 → 8481.90.0000 정정 + 서식 정리
commercial_invoice·packing_list: HS 코드 정정(packing_list는 잔여 SUM 수식
정리 포함). final_invoice·order_confirmation: 서식/속성 정리.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/commercial_invoice.xlsx
+++ b/templates/commercial_invoice.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rotork-my.sharepoint.com/personal/jeongtaek_bang_rotork_com/Documents/바탕 화면/업무/NOAH ACTUATION/noahAutomation/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="107" documentId="11_482B29FEF0C7F80AEE82E0F7E4E761DFCF1F255D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94D4BCAE-56E9-4AC8-B7A0-7A7C39509C3C}"/>
+  <xr:revisionPtr revIDLastSave="119" documentId="11_482B29FEF0C7F80AEE82E0F7E4E761DFCF1F255D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50183257-2972-4614-A95D-9A0DF1678ED1}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="49">
   <si>
     <t>Commercial Invoice</t>
   </si>
@@ -62,9 +62,6 @@
   </si>
   <si>
     <t>Other reference :</t>
-  </si>
-  <si>
-    <t>8481.90.3000</t>
   </si>
   <si>
     <t xml:space="preserve">From  : </t>
@@ -193,6 +190,14 @@
   </si>
   <si>
     <t>PO No.</t>
+    <phoneticPr fontId="17" type="noConversion"/>
+  </si>
+  <si>
+    <t>Currency</t>
+    <phoneticPr fontId="17" type="noConversion"/>
+  </si>
+  <si>
+    <t>8481.90.0000</t>
     <phoneticPr fontId="17" type="noConversion"/>
   </si>
 </sst>
@@ -534,7 +539,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -553,18 +558,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" indent="3" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" indent="3" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -577,16 +573,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -646,18 +636,48 @@
     <xf numFmtId="177" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" indent="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" indent="1" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -785,9 +805,6 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1202,28 +1219,28 @@
   <dimension ref="A1:J42"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.5" style="38" customWidth="1"/>
-    <col min="2" max="2" width="5.6640625" style="38" customWidth="1"/>
-    <col min="3" max="3" width="13.83203125" style="38" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.33203125" style="38" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" style="38" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" style="38" customWidth="1"/>
-    <col min="7" max="7" width="13.83203125" style="38" customWidth="1"/>
-    <col min="8" max="8" width="11.1640625" style="38" customWidth="1"/>
-    <col min="9" max="9" width="21.83203125" style="38" customWidth="1"/>
-    <col min="10" max="10" width="14" style="38" customWidth="1"/>
+    <col min="1" max="1" width="10.5" style="32" customWidth="1"/>
+    <col min="2" max="2" width="5.6640625" style="32" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" style="32" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.33203125" style="32" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" style="32" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" style="32" customWidth="1"/>
+    <col min="7" max="7" width="13.83203125" style="32" customWidth="1"/>
+    <col min="8" max="8" width="11.1640625" style="32" customWidth="1"/>
+    <col min="9" max="9" width="21.83203125" style="32" customWidth="1"/>
+    <col min="10" max="10" width="14" style="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="42"/>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
+      <c r="A1" s="47"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1231,12 +1248,12 @@
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
-      <c r="E2" s="46" t="s">
+      <c r="E2" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
     </row>
@@ -1253,646 +1270,648 @@
       <c r="J3" s="2"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="48" t="s">
+      <c r="A4" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="49"/>
-      <c r="C4" s="49"/>
-      <c r="D4" s="49"/>
-      <c r="E4" s="50"/>
-      <c r="F4" s="28" t="s">
+      <c r="B4" s="54"/>
+      <c r="C4" s="54"/>
+      <c r="D4" s="54"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="G4" s="27"/>
-      <c r="H4" s="17" t="s">
+      <c r="G4" s="22"/>
+      <c r="H4" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="27"/>
+      <c r="I4" s="22"/>
       <c r="J4" s="1"/>
     </row>
     <row r="5" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="58" t="s">
+      <c r="A5" s="63" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="92"/>
+      <c r="C5" s="92"/>
+      <c r="D5" s="92"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="33" t="s">
+        <v>43</v>
+      </c>
+      <c r="G5" s="18"/>
+      <c r="H5" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="I5" s="18"/>
+      <c r="J5" s="1"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" s="94"/>
+      <c r="B6" s="92"/>
+      <c r="C6" s="92"/>
+      <c r="D6" s="92"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="62" t="s">
+        <v>4</v>
+      </c>
+      <c r="G6" s="54"/>
+      <c r="H6" s="54"/>
+      <c r="I6" s="55"/>
+      <c r="J6" s="1"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" s="95"/>
+      <c r="B7" s="96"/>
+      <c r="C7" s="96"/>
+      <c r="D7" s="96"/>
+      <c r="E7" s="97"/>
+      <c r="F7" s="85"/>
+      <c r="G7" s="48"/>
+      <c r="H7" s="48"/>
+      <c r="I7" s="77"/>
+      <c r="J7" s="1"/>
+    </row>
+    <row r="8" spans="1:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="53" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="54"/>
+      <c r="C8" s="54"/>
+      <c r="D8" s="54"/>
+      <c r="E8" s="55"/>
+      <c r="F8" s="86"/>
+      <c r="G8" s="48"/>
+      <c r="H8" s="48"/>
+      <c r="I8" s="77"/>
+      <c r="J8" s="1"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9" s="63"/>
+      <c r="B9" s="64"/>
+      <c r="C9" s="64"/>
+      <c r="D9" s="64"/>
+      <c r="E9" s="65"/>
+      <c r="F9" s="86"/>
+      <c r="G9" s="48"/>
+      <c r="H9" s="48"/>
+      <c r="I9" s="77"/>
+      <c r="J9" s="4"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" s="63"/>
+      <c r="B10" s="64"/>
+      <c r="C10" s="64"/>
+      <c r="D10" s="64"/>
+      <c r="E10" s="65"/>
+      <c r="F10" s="86"/>
+      <c r="G10" s="48"/>
+      <c r="H10" s="48"/>
+      <c r="I10" s="77"/>
+      <c r="J10" s="4"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11" s="66"/>
+      <c r="B11" s="67"/>
+      <c r="C11" s="67"/>
+      <c r="D11" s="67"/>
+      <c r="E11" s="68"/>
+      <c r="F11" s="87"/>
+      <c r="G11" s="59"/>
+      <c r="H11" s="59"/>
+      <c r="I11" s="50"/>
+      <c r="J11" s="2"/>
+    </row>
+    <row r="12" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="53" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" s="54"/>
+      <c r="C12" s="54"/>
+      <c r="D12" s="54"/>
+      <c r="E12" s="55"/>
+      <c r="F12" s="62" t="s">
+        <v>7</v>
+      </c>
+      <c r="G12" s="55"/>
+      <c r="H12" s="89" t="s">
         <v>45</v>
       </c>
-      <c r="B5" s="87"/>
-      <c r="C5" s="87"/>
-      <c r="D5" s="87"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="41" t="s">
-        <v>44</v>
-      </c>
-      <c r="G5" s="23"/>
-      <c r="H5" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="I5" s="23"/>
-      <c r="J5" s="1"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="89"/>
-      <c r="B6" s="87"/>
-      <c r="C6" s="87"/>
-      <c r="D6" s="87"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="57" t="s">
-        <v>4</v>
-      </c>
-      <c r="G6" s="49"/>
-      <c r="H6" s="49"/>
-      <c r="I6" s="50"/>
-      <c r="J6" s="1"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="90"/>
-      <c r="B7" s="91"/>
-      <c r="C7" s="91"/>
-      <c r="D7" s="91"/>
-      <c r="E7" s="92"/>
-      <c r="F7" s="80"/>
-      <c r="G7" s="43"/>
-      <c r="H7" s="43"/>
-      <c r="I7" s="72"/>
-      <c r="J7" s="1"/>
-    </row>
-    <row r="8" spans="1:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="48" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="49"/>
-      <c r="C8" s="49"/>
-      <c r="D8" s="49"/>
-      <c r="E8" s="50"/>
-      <c r="F8" s="81"/>
-      <c r="G8" s="43"/>
-      <c r="H8" s="43"/>
-      <c r="I8" s="72"/>
-      <c r="J8" s="1"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="58"/>
-      <c r="B9" s="59"/>
-      <c r="C9" s="59"/>
-      <c r="D9" s="59"/>
-      <c r="E9" s="60"/>
-      <c r="F9" s="81"/>
-      <c r="G9" s="43"/>
-      <c r="H9" s="43"/>
-      <c r="I9" s="72"/>
-      <c r="J9" s="4"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="58"/>
-      <c r="B10" s="59"/>
-      <c r="C10" s="59"/>
-      <c r="D10" s="59"/>
-      <c r="E10" s="60"/>
-      <c r="F10" s="81"/>
-      <c r="G10" s="43"/>
-      <c r="H10" s="43"/>
-      <c r="I10" s="72"/>
-      <c r="J10" s="4"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="61"/>
-      <c r="B11" s="62"/>
-      <c r="C11" s="62"/>
-      <c r="D11" s="62"/>
-      <c r="E11" s="63"/>
-      <c r="F11" s="82"/>
-      <c r="G11" s="54"/>
-      <c r="H11" s="54"/>
-      <c r="I11" s="45"/>
-      <c r="J11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="48" t="s">
-        <v>6</v>
-      </c>
-      <c r="B12" s="49"/>
-      <c r="C12" s="49"/>
-      <c r="D12" s="49"/>
-      <c r="E12" s="50"/>
-      <c r="F12" s="57" t="s">
-        <v>7</v>
-      </c>
-      <c r="G12" s="50"/>
-      <c r="H12" s="84" t="s">
+      <c r="I12" s="88" t="s">
+        <v>48</v>
+      </c>
+      <c r="J12" s="2"/>
+    </row>
+    <row r="13" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="58"/>
+      <c r="B13" s="59"/>
+      <c r="C13" s="59"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="50"/>
+      <c r="F13" s="86"/>
+      <c r="G13" s="77"/>
+      <c r="H13" s="48"/>
+      <c r="I13" s="77"/>
+      <c r="J13" s="2"/>
+    </row>
+    <row r="14" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14" s="72" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="73"/>
+      <c r="D14" s="73"/>
+      <c r="E14" s="71"/>
+      <c r="F14" s="76" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" s="77"/>
+      <c r="H14" s="48"/>
+      <c r="I14" s="77"/>
+      <c r="J14" s="2"/>
+    </row>
+    <row r="15" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="72"/>
+      <c r="C15" s="73"/>
+      <c r="D15" s="73"/>
+      <c r="E15" s="71"/>
+      <c r="F15" s="49" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="50"/>
+      <c r="H15" s="59"/>
+      <c r="I15" s="50"/>
+      <c r="J15" s="2"/>
+    </row>
+    <row r="16" spans="1:10" ht="17.850000000000001" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="78" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="73"/>
+      <c r="C16" s="73"/>
+      <c r="D16" s="70"/>
+      <c r="E16" s="71"/>
+      <c r="F16" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="G16" s="13"/>
+      <c r="H16" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="I16" s="20"/>
+      <c r="J16" s="1"/>
+    </row>
+    <row r="17" spans="1:10" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="26"/>
+      <c r="B17" s="26"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="31"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="28"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="29"/>
+      <c r="I17" s="30"/>
+      <c r="J17" s="1"/>
+    </row>
+    <row r="18" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="91" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="73"/>
+      <c r="C18" s="73"/>
+      <c r="D18" s="73"/>
+      <c r="E18" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="I12" s="83" t="s">
-        <v>8</v>
-      </c>
-      <c r="J12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="53"/>
-      <c r="B13" s="54"/>
-      <c r="C13" s="54"/>
-      <c r="D13" s="54"/>
-      <c r="E13" s="45"/>
-      <c r="F13" s="81"/>
-      <c r="G13" s="72"/>
-      <c r="H13" s="43"/>
-      <c r="I13" s="72"/>
-      <c r="J13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="B14" s="67" t="s">
-        <v>10</v>
-      </c>
-      <c r="C14" s="68"/>
-      <c r="D14" s="68"/>
-      <c r="E14" s="66"/>
-      <c r="F14" s="71" t="s">
-        <v>11</v>
-      </c>
-      <c r="G14" s="72"/>
-      <c r="H14" s="43"/>
-      <c r="I14" s="72"/>
-      <c r="J14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="29" t="s">
-        <v>12</v>
-      </c>
-      <c r="B15" s="67"/>
-      <c r="C15" s="68"/>
-      <c r="D15" s="68"/>
-      <c r="E15" s="66"/>
-      <c r="F15" s="44" t="s">
-        <v>14</v>
-      </c>
-      <c r="G15" s="45"/>
-      <c r="H15" s="54"/>
-      <c r="I15" s="45"/>
-      <c r="J15" s="2"/>
-    </row>
-    <row r="16" spans="1:10" ht="17.850000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="73" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16" s="68"/>
-      <c r="C16" s="68"/>
-      <c r="D16" s="65"/>
-      <c r="E16" s="66"/>
-      <c r="F16" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="G16" s="18"/>
-      <c r="H16" s="20" t="s">
-        <v>17</v>
-      </c>
-      <c r="I16" s="25"/>
-      <c r="J16" s="1"/>
-    </row>
-    <row r="17" spans="1:10" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="31"/>
-      <c r="B17" s="31"/>
-      <c r="C17" s="31"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="32"/>
-      <c r="F17" s="33"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="34"/>
-      <c r="I17" s="35"/>
-      <c r="J17" s="1"/>
-    </row>
-    <row r="18" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="86" t="s">
+      <c r="F18" s="44" t="s">
         <v>18</v>
       </c>
-      <c r="B18" s="68"/>
-      <c r="C18" s="68"/>
-      <c r="D18" s="68"/>
-      <c r="E18" s="93" t="s">
+      <c r="G18" s="44" t="s">
+        <v>19</v>
+      </c>
+      <c r="H18" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="F18" s="37" t="s">
-        <v>19</v>
-      </c>
-      <c r="G18" s="37" t="s">
+      <c r="I18" s="44" t="s">
         <v>20</v>
       </c>
-      <c r="H18" s="37" t="s">
+      <c r="J18" s="7"/>
+    </row>
+    <row r="19" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="79" t="s">
         <v>21</v>
       </c>
-      <c r="I18" s="37"/>
-      <c r="J18" s="10"/>
-    </row>
-    <row r="19" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="74" t="s">
-        <v>22</v>
-      </c>
-      <c r="B19" s="49"/>
-      <c r="C19" s="49"/>
-      <c r="D19" s="49"/>
+      <c r="B19" s="54"/>
+      <c r="C19" s="54"/>
+      <c r="D19" s="54"/>
       <c r="E19" s="5"/>
       <c r="F19" s="5"/>
       <c r="G19" s="3"/>
-      <c r="H19" s="15"/>
-      <c r="I19" s="15"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="70" t="s">
+      <c r="A20" s="75" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="48"/>
+      <c r="C20" s="48"/>
+      <c r="D20" s="48"/>
+      <c r="E20" s="34"/>
+      <c r="F20" s="39">
+        <v>10</v>
+      </c>
+      <c r="G20" s="37">
+        <v>24</v>
+      </c>
+      <c r="H20" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="43"/>
-      <c r="C20" s="43"/>
-      <c r="D20" s="43"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6">
-        <v>10</v>
-      </c>
-      <c r="G20" s="39">
-        <v>24</v>
-      </c>
-      <c r="H20" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="I20" s="7">
+      <c r="I20" s="6">
         <f t="shared" ref="I20:I27" si="0">E20*G20</f>
         <v>0</v>
       </c>
       <c r="J20" s="1"/>
     </row>
     <row r="21" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="70" t="s">
-        <v>25</v>
-      </c>
-      <c r="B21" s="43"/>
-      <c r="C21" s="43"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6">
+      <c r="A21" s="75" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21" s="48"/>
+      <c r="C21" s="48"/>
+      <c r="D21" s="48"/>
+      <c r="E21" s="34"/>
+      <c r="F21" s="39">
         <v>10</v>
       </c>
-      <c r="G21" s="39">
+      <c r="G21" s="37">
         <v>1.26</v>
       </c>
-      <c r="H21" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="I21" s="7">
+      <c r="H21" s="40" t="s">
+        <v>23</v>
+      </c>
+      <c r="I21" s="6">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="J21" s="1"/>
     </row>
     <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="70" t="s">
-        <v>26</v>
-      </c>
-      <c r="B22" s="43"/>
-      <c r="C22" s="43"/>
-      <c r="D22" s="43"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6">
+      <c r="A22" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="B22" s="48"/>
+      <c r="C22" s="48"/>
+      <c r="D22" s="48"/>
+      <c r="E22" s="34"/>
+      <c r="F22" s="39">
         <v>10</v>
       </c>
-      <c r="G22" s="39">
+      <c r="G22" s="37">
         <v>3.7</v>
       </c>
-      <c r="H22" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="I22" s="7">
+      <c r="H22" s="40" t="s">
+        <v>23</v>
+      </c>
+      <c r="I22" s="6">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="J22" s="1"/>
     </row>
     <row r="23" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="70" t="s">
-        <v>27</v>
-      </c>
-      <c r="B23" s="43"/>
-      <c r="C23" s="43"/>
-      <c r="D23" s="43"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6">
+      <c r="A23" s="75" t="s">
+        <v>26</v>
+      </c>
+      <c r="B23" s="48"/>
+      <c r="C23" s="48"/>
+      <c r="D23" s="48"/>
+      <c r="E23" s="34"/>
+      <c r="F23" s="39">
         <v>10</v>
       </c>
-      <c r="G23" s="39">
+      <c r="G23" s="37">
         <v>3.9</v>
       </c>
-      <c r="H23" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="I23" s="7">
+      <c r="H23" s="40" t="s">
+        <v>23</v>
+      </c>
+      <c r="I23" s="6">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="J23" s="1"/>
     </row>
     <row r="24" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="70" t="s">
-        <v>28</v>
-      </c>
-      <c r="B24" s="43"/>
-      <c r="C24" s="43"/>
-      <c r="D24" s="43"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6">
+      <c r="A24" s="75" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" s="48"/>
+      <c r="C24" s="48"/>
+      <c r="D24" s="48"/>
+      <c r="E24" s="34"/>
+      <c r="F24" s="39">
         <v>10</v>
       </c>
-      <c r="G24" s="39">
+      <c r="G24" s="37">
         <v>3.9</v>
       </c>
-      <c r="H24" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="I24" s="7">
+      <c r="H24" s="40" t="s">
+        <v>23</v>
+      </c>
+      <c r="I24" s="6">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="J24" s="1"/>
     </row>
     <row r="25" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="70" t="s">
-        <v>29</v>
-      </c>
-      <c r="B25" s="43"/>
-      <c r="C25" s="43"/>
-      <c r="D25" s="43"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6">
+      <c r="A25" s="75" t="s">
+        <v>28</v>
+      </c>
+      <c r="B25" s="48"/>
+      <c r="C25" s="48"/>
+      <c r="D25" s="48"/>
+      <c r="E25" s="34"/>
+      <c r="F25" s="39">
         <v>10</v>
       </c>
-      <c r="G25" s="39">
+      <c r="G25" s="37">
         <v>2.5</v>
       </c>
-      <c r="H25" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="I25" s="7">
+      <c r="H25" s="40" t="s">
+        <v>23</v>
+      </c>
+      <c r="I25" s="6">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="J25" s="1"/>
     </row>
     <row r="26" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="70" t="s">
-        <v>30</v>
-      </c>
-      <c r="B26" s="43"/>
-      <c r="C26" s="43"/>
-      <c r="D26" s="43"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6">
+      <c r="A26" s="75" t="s">
+        <v>29</v>
+      </c>
+      <c r="B26" s="48"/>
+      <c r="C26" s="48"/>
+      <c r="D26" s="48"/>
+      <c r="E26" s="34"/>
+      <c r="F26" s="39">
         <v>10</v>
       </c>
-      <c r="G26" s="39">
+      <c r="G26" s="37">
         <v>2.9</v>
       </c>
-      <c r="H26" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="I26" s="7">
+      <c r="H26" s="40" t="s">
+        <v>23</v>
+      </c>
+      <c r="I26" s="6">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="J26" s="1"/>
     </row>
     <row r="27" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="69" t="s">
-        <v>31</v>
-      </c>
-      <c r="B27" s="54"/>
-      <c r="C27" s="54"/>
-      <c r="D27" s="54"/>
-      <c r="E27" s="8"/>
-      <c r="F27" s="8">
+      <c r="A27" s="74" t="s">
+        <v>30</v>
+      </c>
+      <c r="B27" s="59"/>
+      <c r="C27" s="59"/>
+      <c r="D27" s="59"/>
+      <c r="E27" s="35"/>
+      <c r="F27" s="41">
         <v>10</v>
       </c>
-      <c r="G27" s="40">
+      <c r="G27" s="38">
         <v>2.9</v>
       </c>
-      <c r="H27" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="I27" s="7">
+      <c r="H27" s="42" t="s">
+        <v>23</v>
+      </c>
+      <c r="I27" s="6">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="J27" s="1"/>
     </row>
     <row r="28" spans="1:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="51" t="s">
-        <v>32</v>
-      </c>
-      <c r="B28" s="52"/>
-      <c r="C28" s="52"/>
-      <c r="D28" s="52"/>
-      <c r="E28" s="21"/>
-      <c r="F28" s="21">
+      <c r="A28" s="56" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" s="57"/>
+      <c r="C28" s="57"/>
+      <c r="D28" s="57"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="43">
         <f>SUM(F20:F27)</f>
         <v>80</v>
       </c>
-      <c r="G28" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="H28" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="I28" s="30">
+      <c r="G28" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="H28" s="36" t="s">
+        <v>23</v>
+      </c>
+      <c r="I28" s="25">
         <f>SUM(I20:I27)</f>
         <v>0</v>
       </c>
       <c r="J28" s="2"/>
     </row>
     <row r="29" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="55" t="s">
+      <c r="A29" s="60" t="s">
+        <v>33</v>
+      </c>
+      <c r="B29" s="61"/>
+      <c r="C29" s="61"/>
+      <c r="D29" s="61"/>
+      <c r="E29" s="61"/>
+      <c r="F29" s="61"/>
+      <c r="G29" s="61"/>
+      <c r="H29" s="61"/>
+      <c r="I29" s="61"/>
+      <c r="J29" s="7"/>
+    </row>
+    <row r="30" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="21"/>
+      <c r="B30" s="21"/>
+      <c r="C30" s="21"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="21"/>
+      <c r="H30" s="21"/>
+      <c r="I30" s="21"/>
+      <c r="J30" s="7"/>
+    </row>
+    <row r="31" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="80" t="s">
         <v>34</v>
       </c>
-      <c r="B29" s="56"/>
-      <c r="C29" s="56"/>
-      <c r="D29" s="56"/>
-      <c r="E29" s="56"/>
-      <c r="F29" s="56"/>
-      <c r="G29" s="56"/>
-      <c r="H29" s="56"/>
-      <c r="I29" s="56"/>
-      <c r="J29" s="10"/>
-    </row>
-    <row r="30" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="26"/>
-      <c r="B30" s="26"/>
-      <c r="C30" s="26"/>
-      <c r="D30" s="26"/>
-      <c r="E30" s="26"/>
-      <c r="F30" s="26"/>
-      <c r="G30" s="26"/>
-      <c r="H30" s="26"/>
-      <c r="I30" s="26"/>
-      <c r="J30" s="10"/>
-    </row>
-    <row r="31" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="75" t="s">
+      <c r="B31" s="48"/>
+      <c r="C31" s="48"/>
+      <c r="D31" s="48"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="21"/>
+      <c r="G31" s="21"/>
+      <c r="H31" s="21"/>
+      <c r="I31" s="21"/>
+      <c r="J31" s="7"/>
+    </row>
+    <row r="32" spans="1:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="80" t="s">
         <v>35</v>
       </c>
-      <c r="B31" s="43"/>
-      <c r="C31" s="43"/>
-      <c r="D31" s="43"/>
-      <c r="E31" s="26"/>
-      <c r="F31" s="26"/>
-      <c r="G31" s="26"/>
-      <c r="H31" s="26"/>
-      <c r="I31" s="26"/>
-      <c r="J31" s="10"/>
-    </row>
-    <row r="32" spans="1:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="75" t="s">
+      <c r="B32" s="48"/>
+      <c r="C32" s="48"/>
+      <c r="D32" s="48"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="21"/>
+      <c r="G32" s="21"/>
+      <c r="H32" s="21"/>
+      <c r="I32" s="21"/>
+      <c r="J32" s="7"/>
+    </row>
+    <row r="33" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="81" t="s">
+        <v>12</v>
+      </c>
+      <c r="B33" s="82"/>
+      <c r="C33" s="82"/>
+      <c r="D33" s="82"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="21"/>
+      <c r="G33" s="21"/>
+      <c r="H33" s="21"/>
+      <c r="I33" s="21"/>
+      <c r="J33" s="7"/>
+    </row>
+    <row r="34" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="52" t="s">
         <v>36</v>
       </c>
-      <c r="B32" s="43"/>
-      <c r="C32" s="43"/>
-      <c r="D32" s="43"/>
-      <c r="E32" s="26"/>
-      <c r="F32" s="26"/>
-      <c r="G32" s="26"/>
-      <c r="H32" s="26"/>
-      <c r="I32" s="26"/>
-      <c r="J32" s="10"/>
-    </row>
-    <row r="33" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="76" t="s">
-        <v>13</v>
-      </c>
-      <c r="B33" s="77"/>
-      <c r="C33" s="77"/>
-      <c r="D33" s="77"/>
-      <c r="E33" s="26"/>
-      <c r="F33" s="26"/>
-      <c r="G33" s="26"/>
-      <c r="H33" s="26"/>
-      <c r="I33" s="26"/>
-      <c r="J33" s="10"/>
-    </row>
-    <row r="34" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="47" t="s">
+      <c r="B34" s="48"/>
+      <c r="C34" s="52">
+        <v>8116409</v>
+      </c>
+      <c r="D34" s="48"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="8"/>
+      <c r="H34" s="8"/>
+      <c r="I34" s="8"/>
+      <c r="J34" s="9"/>
+    </row>
+    <row r="35" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="52" t="s">
         <v>37</v>
       </c>
-      <c r="B34" s="43"/>
-      <c r="C34" s="47">
-        <v>8116409</v>
-      </c>
-      <c r="D34" s="43"/>
-      <c r="E34" s="11"/>
-      <c r="F34" s="11"/>
-      <c r="G34" s="11"/>
-      <c r="H34" s="11"/>
-      <c r="I34" s="11"/>
-      <c r="J34" s="12"/>
-    </row>
-    <row r="35" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="47" t="s">
+      <c r="B35" s="48"/>
+      <c r="C35" s="90"/>
+      <c r="D35" s="48"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="8"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="8"/>
+      <c r="I35" s="8"/>
+      <c r="J35" s="9"/>
+    </row>
+    <row r="36" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="43"/>
-      <c r="C35" s="85"/>
-      <c r="D35" s="43"/>
-      <c r="E35" s="11"/>
-      <c r="F35" s="11"/>
-      <c r="G35" s="11"/>
-      <c r="H35" s="11"/>
-      <c r="I35" s="11"/>
-      <c r="J35" s="12"/>
-    </row>
-    <row r="36" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="47" t="s">
+      <c r="B36" s="48"/>
+      <c r="C36" s="80"/>
+      <c r="D36" s="48"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="8"/>
+      <c r="H36" s="8"/>
+      <c r="I36" s="8"/>
+      <c r="J36" s="9"/>
+    </row>
+    <row r="37" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="19"/>
+      <c r="B37" s="19"/>
+      <c r="C37" s="19"/>
+      <c r="D37" s="19"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8"/>
+      <c r="G37" s="8"/>
+      <c r="H37" s="8"/>
+      <c r="I37" s="8"/>
+      <c r="J37" s="9"/>
+    </row>
+    <row r="38" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="19"/>
+      <c r="B38" s="19"/>
+      <c r="C38" s="19"/>
+      <c r="D38" s="19"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="8"/>
+      <c r="H38" s="8"/>
+      <c r="I38" s="8"/>
+      <c r="J38" s="9"/>
+    </row>
+    <row r="39" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="19"/>
+      <c r="B39" s="19"/>
+      <c r="C39" s="19"/>
+      <c r="D39" s="19"/>
+      <c r="E39" s="8"/>
+      <c r="F39" s="8"/>
+      <c r="G39" s="8"/>
+      <c r="H39" s="8"/>
+      <c r="I39" s="8"/>
+      <c r="J39" s="9"/>
+    </row>
+    <row r="40" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="19"/>
+      <c r="B40" s="19"/>
+      <c r="C40" s="19"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="8"/>
+      <c r="F40" s="8"/>
+      <c r="G40" s="8"/>
+      <c r="H40" s="8"/>
+      <c r="I40" s="8"/>
+      <c r="J40" s="9"/>
+    </row>
+    <row r="41" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="84" t="s">
         <v>39</v>
       </c>
-      <c r="B36" s="43"/>
-      <c r="C36" s="75"/>
-      <c r="D36" s="43"/>
-      <c r="E36" s="11"/>
-      <c r="F36" s="11"/>
-      <c r="G36" s="11"/>
-      <c r="H36" s="11"/>
-      <c r="I36" s="11"/>
-      <c r="J36" s="12"/>
-    </row>
-    <row r="37" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="24"/>
-      <c r="B37" s="24"/>
-      <c r="C37" s="24"/>
-      <c r="D37" s="24"/>
-      <c r="E37" s="11"/>
-      <c r="F37" s="11"/>
-      <c r="G37" s="11"/>
-      <c r="H37" s="11"/>
-      <c r="I37" s="11"/>
-      <c r="J37" s="12"/>
-    </row>
-    <row r="38" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="24"/>
-      <c r="B38" s="24"/>
-      <c r="C38" s="24"/>
-      <c r="D38" s="24"/>
-      <c r="E38" s="11"/>
-      <c r="F38" s="11"/>
-      <c r="G38" s="11"/>
-      <c r="H38" s="11"/>
-      <c r="I38" s="11"/>
-      <c r="J38" s="12"/>
-    </row>
-    <row r="39" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="24"/>
-      <c r="B39" s="24"/>
-      <c r="C39" s="24"/>
-      <c r="D39" s="24"/>
-      <c r="E39" s="11"/>
-      <c r="F39" s="11"/>
-      <c r="G39" s="11"/>
-      <c r="H39" s="11"/>
-      <c r="I39" s="11"/>
-      <c r="J39" s="12"/>
-    </row>
-    <row r="40" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="24"/>
-      <c r="B40" s="24"/>
-      <c r="C40" s="24"/>
-      <c r="D40" s="24"/>
-      <c r="E40" s="11"/>
-      <c r="F40" s="11"/>
-      <c r="G40" s="11"/>
-      <c r="H40" s="11"/>
-      <c r="I40" s="11"/>
-      <c r="J40" s="12"/>
-    </row>
-    <row r="41" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="79" t="s">
+      <c r="B41" s="48"/>
+      <c r="C41" s="48"/>
+      <c r="D41" s="48"/>
+      <c r="E41" s="48"/>
+      <c r="F41" s="48"/>
+      <c r="G41" s="48"/>
+      <c r="H41" s="48"/>
+      <c r="I41" s="48"/>
+      <c r="J41" s="9"/>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A42" s="83" t="s">
         <v>40</v>
       </c>
-      <c r="B41" s="43"/>
-      <c r="C41" s="43"/>
-      <c r="D41" s="43"/>
-      <c r="E41" s="43"/>
-      <c r="F41" s="43"/>
-      <c r="G41" s="43"/>
-      <c r="H41" s="43"/>
-      <c r="I41" s="43"/>
-      <c r="J41" s="12"/>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A42" s="78" t="s">
+      <c r="B42" s="48"/>
+      <c r="C42" s="48"/>
+      <c r="D42" s="48"/>
+      <c r="E42" s="48"/>
+      <c r="F42" s="69" t="s">
         <v>41</v>
       </c>
-      <c r="B42" s="43"/>
-      <c r="C42" s="43"/>
-      <c r="D42" s="43"/>
-      <c r="E42" s="43"/>
-      <c r="F42" s="64" t="s">
-        <v>42</v>
-      </c>
-      <c r="G42" s="43"/>
-      <c r="H42" s="43"/>
-      <c r="I42" s="43"/>
-      <c r="J42" s="13"/>
+      <c r="G42" s="48"/>
+      <c r="H42" s="48"/>
+      <c r="I42" s="48"/>
+      <c r="J42" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="45">

</xml_diff>

<commit_message>
chore(templates): CI/FI/PL 서식 수정 반영 (2026-07-14~22 작업분)
문서를 뽑으며 손본 서식이 템플릿에 남아 있었는데 기록 없이 미커밋 상태였다.
무슨 변경인지는 xlsx 내부(styles.xml / sheet1.xml)를 열어 확인했다.

- commercial_invoice (7/22) — 숫자서식 4→6종 추가
  (`#,##0.00_ `, 음수 빨강 괄호 `0_);[Red]\(0\)` 등), 열 너비 조정
- final_invoice (7/15) — 숫자서식 추가, 셀 스타일 교체(A1 s=46→37),
  일부 셀의 정렬·들여쓰기 제거
- packing_list (7/14) — 회계 숫자서식 `_-* #,##0.0_-;...` 1종 제거, 셀 스타일 다수 변경

셀 매핑(어느 칸에 무엇이 들어가는지)은 바뀌지 않아 `create_ci/fi/pl.py`는 그대로 동작한다.
`docs/TEMPLATE_MAPPINGS.md`도 수정할 것이 없다.

커서 위치·창 크기·저장 경로(packing_list: SharePoint URL → 로컬 경로)도 함께 들어갔는데,
이건 Excel이 저장하며 붙인 것이라 의미 없다.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/commercial_invoice.xlsx
+++ b/templates/commercial_invoice.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rotork-my.sharepoint.com/personal/jeongtaek_bang_rotork_com/Documents/바탕 화면/업무/NOAH ACTUATION/noahAutomation/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="119" documentId="11_482B29FEF0C7F80AEE82E0F7E4E761DFCF1F255D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50183257-2972-4614-A95D-9A0DF1678ED1}"/>
+  <xr:revisionPtr revIDLastSave="128" documentId="11_482B29FEF0C7F80AEE82E0F7E4E761DFCF1F255D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{003538BF-ABC0-4566-B951-8AABCECF7593}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -205,11 +205,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="4">
+  <numFmts count="6">
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="176" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="177" formatCode="yyyy\-mm\-dd;@"/>
-    <numFmt numFmtId="178" formatCode="0.00_ "/>
+    <numFmt numFmtId="179" formatCode="0_);[Red]\(0\)"/>
+    <numFmt numFmtId="181" formatCode="#,##0.00_ "/>
+    <numFmt numFmtId="182" formatCode="#,##0.00_);[Red]\(#,##0.00\)"/>
   </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
@@ -558,9 +560,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -649,27 +648,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -678,6 +662,15 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="179" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="179" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="179" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -805,6 +798,15 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="182" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1219,28 +1221,28 @@
   <dimension ref="A1:J42"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.5" style="32" customWidth="1"/>
-    <col min="2" max="2" width="5.6640625" style="32" customWidth="1"/>
-    <col min="3" max="3" width="13.83203125" style="32" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.33203125" style="32" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" style="32" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" style="32" customWidth="1"/>
-    <col min="7" max="7" width="13.83203125" style="32" customWidth="1"/>
-    <col min="8" max="8" width="11.1640625" style="32" customWidth="1"/>
-    <col min="9" max="9" width="21.83203125" style="32" customWidth="1"/>
-    <col min="10" max="10" width="14" style="32" customWidth="1"/>
+    <col min="1" max="1" width="10.5" style="31" customWidth="1"/>
+    <col min="2" max="2" width="5.6640625" style="31" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" style="31" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.33203125" style="31" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" style="31" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" style="31" customWidth="1"/>
+    <col min="7" max="7" width="13.83203125" style="31" customWidth="1"/>
+    <col min="8" max="8" width="11.1640625" style="31" customWidth="1"/>
+    <col min="9" max="9" width="21.83203125" style="31" customWidth="1"/>
+    <col min="10" max="10" width="14" style="31" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="47"/>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
+      <c r="A1" s="44"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1248,12 +1250,12 @@
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
-      <c r="E2" s="51" t="s">
+      <c r="E2" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
     </row>
@@ -1270,648 +1272,648 @@
       <c r="J3" s="2"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="53" t="s">
+      <c r="A4" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="54"/>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="23" t="s">
+      <c r="B4" s="51"/>
+      <c r="C4" s="51"/>
+      <c r="D4" s="51"/>
+      <c r="E4" s="52"/>
+      <c r="F4" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="G4" s="22"/>
-      <c r="H4" s="12" t="s">
+      <c r="G4" s="21"/>
+      <c r="H4" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="22"/>
+      <c r="I4" s="21"/>
       <c r="J4" s="1"/>
     </row>
     <row r="5" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="63" t="s">
+      <c r="A5" s="60" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="92"/>
-      <c r="C5" s="92"/>
-      <c r="D5" s="92"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="33" t="s">
+      <c r="B5" s="89"/>
+      <c r="C5" s="89"/>
+      <c r="D5" s="89"/>
+      <c r="E5" s="90"/>
+      <c r="F5" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="G5" s="18"/>
-      <c r="H5" s="14" t="s">
+      <c r="G5" s="17"/>
+      <c r="H5" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="I5" s="18"/>
+      <c r="I5" s="17"/>
       <c r="J5" s="1"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="94"/>
-      <c r="B6" s="92"/>
-      <c r="C6" s="92"/>
-      <c r="D6" s="92"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="62" t="s">
+      <c r="A6" s="91"/>
+      <c r="B6" s="89"/>
+      <c r="C6" s="89"/>
+      <c r="D6" s="89"/>
+      <c r="E6" s="90"/>
+      <c r="F6" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="54"/>
-      <c r="H6" s="54"/>
-      <c r="I6" s="55"/>
+      <c r="G6" s="51"/>
+      <c r="H6" s="51"/>
+      <c r="I6" s="52"/>
       <c r="J6" s="1"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="95"/>
-      <c r="B7" s="96"/>
-      <c r="C7" s="96"/>
-      <c r="D7" s="96"/>
-      <c r="E7" s="97"/>
-      <c r="F7" s="85"/>
-      <c r="G7" s="48"/>
-      <c r="H7" s="48"/>
-      <c r="I7" s="77"/>
+      <c r="A7" s="92"/>
+      <c r="B7" s="93"/>
+      <c r="C7" s="93"/>
+      <c r="D7" s="93"/>
+      <c r="E7" s="94"/>
+      <c r="F7" s="82"/>
+      <c r="G7" s="45"/>
+      <c r="H7" s="45"/>
+      <c r="I7" s="74"/>
       <c r="J7" s="1"/>
     </row>
     <row r="8" spans="1:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="53" t="s">
+      <c r="A8" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="54"/>
-      <c r="C8" s="54"/>
-      <c r="D8" s="54"/>
-      <c r="E8" s="55"/>
-      <c r="F8" s="86"/>
-      <c r="G8" s="48"/>
-      <c r="H8" s="48"/>
-      <c r="I8" s="77"/>
+      <c r="B8" s="51"/>
+      <c r="C8" s="51"/>
+      <c r="D8" s="51"/>
+      <c r="E8" s="52"/>
+      <c r="F8" s="83"/>
+      <c r="G8" s="45"/>
+      <c r="H8" s="45"/>
+      <c r="I8" s="74"/>
       <c r="J8" s="1"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="63"/>
-      <c r="B9" s="64"/>
-      <c r="C9" s="64"/>
-      <c r="D9" s="64"/>
-      <c r="E9" s="65"/>
-      <c r="F9" s="86"/>
-      <c r="G9" s="48"/>
-      <c r="H9" s="48"/>
-      <c r="I9" s="77"/>
+      <c r="A9" s="60"/>
+      <c r="B9" s="61"/>
+      <c r="C9" s="61"/>
+      <c r="D9" s="61"/>
+      <c r="E9" s="62"/>
+      <c r="F9" s="83"/>
+      <c r="G9" s="45"/>
+      <c r="H9" s="45"/>
+      <c r="I9" s="74"/>
       <c r="J9" s="4"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="63"/>
-      <c r="B10" s="64"/>
-      <c r="C10" s="64"/>
-      <c r="D10" s="64"/>
-      <c r="E10" s="65"/>
-      <c r="F10" s="86"/>
-      <c r="G10" s="48"/>
-      <c r="H10" s="48"/>
-      <c r="I10" s="77"/>
+      <c r="A10" s="60"/>
+      <c r="B10" s="61"/>
+      <c r="C10" s="61"/>
+      <c r="D10" s="61"/>
+      <c r="E10" s="62"/>
+      <c r="F10" s="83"/>
+      <c r="G10" s="45"/>
+      <c r="H10" s="45"/>
+      <c r="I10" s="74"/>
       <c r="J10" s="4"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="66"/>
-      <c r="B11" s="67"/>
-      <c r="C11" s="67"/>
-      <c r="D11" s="67"/>
-      <c r="E11" s="68"/>
-      <c r="F11" s="87"/>
-      <c r="G11" s="59"/>
-      <c r="H11" s="59"/>
-      <c r="I11" s="50"/>
+      <c r="A11" s="63"/>
+      <c r="B11" s="64"/>
+      <c r="C11" s="64"/>
+      <c r="D11" s="64"/>
+      <c r="E11" s="65"/>
+      <c r="F11" s="84"/>
+      <c r="G11" s="56"/>
+      <c r="H11" s="56"/>
+      <c r="I11" s="47"/>
       <c r="J11" s="2"/>
     </row>
     <row r="12" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="53" t="s">
+      <c r="A12" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="54"/>
-      <c r="C12" s="54"/>
-      <c r="D12" s="54"/>
-      <c r="E12" s="55"/>
-      <c r="F12" s="62" t="s">
+      <c r="B12" s="51"/>
+      <c r="C12" s="51"/>
+      <c r="D12" s="51"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="59" t="s">
         <v>7</v>
       </c>
-      <c r="G12" s="55"/>
-      <c r="H12" s="89" t="s">
+      <c r="G12" s="52"/>
+      <c r="H12" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="I12" s="88" t="s">
+      <c r="I12" s="85" t="s">
         <v>48</v>
       </c>
       <c r="J12" s="2"/>
     </row>
     <row r="13" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="58"/>
-      <c r="B13" s="59"/>
-      <c r="C13" s="59"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="50"/>
-      <c r="F13" s="86"/>
-      <c r="G13" s="77"/>
-      <c r="H13" s="48"/>
-      <c r="I13" s="77"/>
+      <c r="A13" s="55"/>
+      <c r="B13" s="56"/>
+      <c r="C13" s="56"/>
+      <c r="D13" s="56"/>
+      <c r="E13" s="47"/>
+      <c r="F13" s="83"/>
+      <c r="G13" s="74"/>
+      <c r="H13" s="45"/>
+      <c r="I13" s="74"/>
       <c r="J13" s="2"/>
     </row>
     <row r="14" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="24" t="s">
+      <c r="A14" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="72" t="s">
+      <c r="B14" s="69" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="73"/>
-      <c r="D14" s="73"/>
-      <c r="E14" s="71"/>
-      <c r="F14" s="76" t="s">
+      <c r="C14" s="70"/>
+      <c r="D14" s="70"/>
+      <c r="E14" s="68"/>
+      <c r="F14" s="73" t="s">
         <v>10</v>
       </c>
-      <c r="G14" s="77"/>
-      <c r="H14" s="48"/>
-      <c r="I14" s="77"/>
+      <c r="G14" s="74"/>
+      <c r="H14" s="45"/>
+      <c r="I14" s="74"/>
       <c r="J14" s="2"/>
     </row>
     <row r="15" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="24" t="s">
+      <c r="A15" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="B15" s="72"/>
-      <c r="C15" s="73"/>
-      <c r="D15" s="73"/>
-      <c r="E15" s="71"/>
-      <c r="F15" s="49" t="s">
+      <c r="B15" s="69"/>
+      <c r="C15" s="70"/>
+      <c r="D15" s="70"/>
+      <c r="E15" s="68"/>
+      <c r="F15" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="G15" s="50"/>
-      <c r="H15" s="59"/>
-      <c r="I15" s="50"/>
+      <c r="G15" s="47"/>
+      <c r="H15" s="56"/>
+      <c r="I15" s="47"/>
       <c r="J15" s="2"/>
     </row>
     <row r="16" spans="1:10" ht="17.850000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="78" t="s">
+      <c r="A16" s="75" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="73"/>
-      <c r="C16" s="73"/>
-      <c r="D16" s="70"/>
-      <c r="E16" s="71"/>
-      <c r="F16" s="17" t="s">
+      <c r="B16" s="70"/>
+      <c r="C16" s="70"/>
+      <c r="D16" s="67"/>
+      <c r="E16" s="68"/>
+      <c r="F16" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="G16" s="13"/>
-      <c r="H16" s="15" t="s">
+      <c r="G16" s="12"/>
+      <c r="H16" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="I16" s="20"/>
+      <c r="I16" s="19"/>
       <c r="J16" s="1"/>
     </row>
     <row r="17" spans="1:10" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="26"/>
-      <c r="B17" s="26"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="31"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="28"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="29"/>
-      <c r="I17" s="30"/>
+      <c r="A17" s="25"/>
+      <c r="B17" s="25"/>
+      <c r="C17" s="25"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="28"/>
+      <c r="I17" s="29"/>
       <c r="J17" s="1"/>
     </row>
     <row r="18" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="91" t="s">
+      <c r="A18" s="88" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="73"/>
-      <c r="C18" s="73"/>
-      <c r="D18" s="73"/>
-      <c r="E18" s="45" t="s">
+      <c r="B18" s="70"/>
+      <c r="C18" s="70"/>
+      <c r="D18" s="70"/>
+      <c r="E18" s="39" t="s">
         <v>46</v>
       </c>
-      <c r="F18" s="44" t="s">
+      <c r="F18" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="G18" s="44" t="s">
+      <c r="G18" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="H18" s="46" t="s">
+      <c r="H18" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="I18" s="44" t="s">
+      <c r="I18" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="J18" s="7"/>
+      <c r="J18" s="6"/>
     </row>
     <row r="19" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="79" t="s">
+      <c r="A19" s="76" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="54"/>
-      <c r="C19" s="54"/>
-      <c r="D19" s="54"/>
+      <c r="B19" s="51"/>
+      <c r="C19" s="51"/>
+      <c r="D19" s="51"/>
       <c r="E19" s="5"/>
       <c r="F19" s="5"/>
       <c r="G19" s="3"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="11"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="75" t="s">
+      <c r="A20" s="72" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="48"/>
-      <c r="C20" s="48"/>
-      <c r="D20" s="48"/>
-      <c r="E20" s="34"/>
-      <c r="F20" s="39">
+      <c r="B20" s="45"/>
+      <c r="C20" s="45"/>
+      <c r="D20" s="45"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="41">
         <v>10</v>
       </c>
-      <c r="G20" s="37">
+      <c r="G20" s="95">
         <v>24</v>
       </c>
-      <c r="H20" s="40" t="s">
+      <c r="H20" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="I20" s="6">
+      <c r="I20" s="97">
         <f t="shared" ref="I20:I27" si="0">E20*G20</f>
         <v>0</v>
       </c>
       <c r="J20" s="1"/>
     </row>
     <row r="21" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="75" t="s">
+      <c r="A21" s="72" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="48"/>
-      <c r="C21" s="48"/>
-      <c r="D21" s="48"/>
-      <c r="E21" s="34"/>
-      <c r="F21" s="39">
+      <c r="B21" s="45"/>
+      <c r="C21" s="45"/>
+      <c r="D21" s="45"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="41">
         <v>10</v>
       </c>
-      <c r="G21" s="37">
+      <c r="G21" s="95">
         <v>1.26</v>
       </c>
-      <c r="H21" s="40" t="s">
+      <c r="H21" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="I21" s="6">
+      <c r="I21" s="97">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="J21" s="1"/>
     </row>
     <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="75" t="s">
+      <c r="A22" s="72" t="s">
         <v>25</v>
       </c>
-      <c r="B22" s="48"/>
-      <c r="C22" s="48"/>
-      <c r="D22" s="48"/>
-      <c r="E22" s="34"/>
-      <c r="F22" s="39">
+      <c r="B22" s="45"/>
+      <c r="C22" s="45"/>
+      <c r="D22" s="45"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="41">
         <v>10</v>
       </c>
-      <c r="G22" s="37">
+      <c r="G22" s="95">
         <v>3.7</v>
       </c>
-      <c r="H22" s="40" t="s">
+      <c r="H22" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="I22" s="6">
+      <c r="I22" s="97">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="J22" s="1"/>
     </row>
     <row r="23" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="75" t="s">
+      <c r="A23" s="72" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="48"/>
-      <c r="C23" s="48"/>
-      <c r="D23" s="48"/>
-      <c r="E23" s="34"/>
-      <c r="F23" s="39">
+      <c r="B23" s="45"/>
+      <c r="C23" s="45"/>
+      <c r="D23" s="45"/>
+      <c r="E23" s="33"/>
+      <c r="F23" s="41">
         <v>10</v>
       </c>
-      <c r="G23" s="37">
+      <c r="G23" s="95">
         <v>3.9</v>
       </c>
-      <c r="H23" s="40" t="s">
+      <c r="H23" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="I23" s="6">
+      <c r="I23" s="97">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="J23" s="1"/>
     </row>
     <row r="24" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="75" t="s">
+      <c r="A24" s="72" t="s">
         <v>27</v>
       </c>
-      <c r="B24" s="48"/>
-      <c r="C24" s="48"/>
-      <c r="D24" s="48"/>
-      <c r="E24" s="34"/>
-      <c r="F24" s="39">
+      <c r="B24" s="45"/>
+      <c r="C24" s="45"/>
+      <c r="D24" s="45"/>
+      <c r="E24" s="33"/>
+      <c r="F24" s="41">
         <v>10</v>
       </c>
-      <c r="G24" s="37">
+      <c r="G24" s="95">
         <v>3.9</v>
       </c>
-      <c r="H24" s="40" t="s">
+      <c r="H24" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="I24" s="6">
+      <c r="I24" s="97">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="J24" s="1"/>
     </row>
     <row r="25" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="75" t="s">
+      <c r="A25" s="72" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="48"/>
-      <c r="C25" s="48"/>
-      <c r="D25" s="48"/>
-      <c r="E25" s="34"/>
-      <c r="F25" s="39">
+      <c r="B25" s="45"/>
+      <c r="C25" s="45"/>
+      <c r="D25" s="45"/>
+      <c r="E25" s="33"/>
+      <c r="F25" s="41">
         <v>10</v>
       </c>
-      <c r="G25" s="37">
+      <c r="G25" s="95">
         <v>2.5</v>
       </c>
-      <c r="H25" s="40" t="s">
+      <c r="H25" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="I25" s="6">
+      <c r="I25" s="97">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="J25" s="1"/>
     </row>
     <row r="26" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="75" t="s">
+      <c r="A26" s="72" t="s">
         <v>29</v>
       </c>
-      <c r="B26" s="48"/>
-      <c r="C26" s="48"/>
-      <c r="D26" s="48"/>
-      <c r="E26" s="34"/>
-      <c r="F26" s="39">
+      <c r="B26" s="45"/>
+      <c r="C26" s="45"/>
+      <c r="D26" s="45"/>
+      <c r="E26" s="33"/>
+      <c r="F26" s="41">
         <v>10</v>
       </c>
-      <c r="G26" s="37">
+      <c r="G26" s="95">
         <v>2.9</v>
       </c>
-      <c r="H26" s="40" t="s">
+      <c r="H26" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="I26" s="6">
+      <c r="I26" s="97">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="J26" s="1"/>
     </row>
     <row r="27" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="74" t="s">
+      <c r="A27" s="71" t="s">
         <v>30</v>
       </c>
-      <c r="B27" s="59"/>
-      <c r="C27" s="59"/>
-      <c r="D27" s="59"/>
-      <c r="E27" s="35"/>
-      <c r="F27" s="41">
+      <c r="B27" s="56"/>
+      <c r="C27" s="56"/>
+      <c r="D27" s="56"/>
+      <c r="E27" s="34"/>
+      <c r="F27" s="42">
         <v>10</v>
       </c>
-      <c r="G27" s="38">
+      <c r="G27" s="96">
         <v>2.9</v>
       </c>
-      <c r="H27" s="42" t="s">
+      <c r="H27" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="I27" s="6">
+      <c r="I27" s="97">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="J27" s="1"/>
     </row>
     <row r="28" spans="1:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="56" t="s">
+      <c r="A28" s="53" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="57"/>
-      <c r="C28" s="57"/>
-      <c r="D28" s="57"/>
-      <c r="E28" s="16"/>
+      <c r="B28" s="54"/>
+      <c r="C28" s="54"/>
+      <c r="D28" s="54"/>
+      <c r="E28" s="15"/>
       <c r="F28" s="43">
         <f>SUM(F20:F27)</f>
         <v>80</v>
       </c>
-      <c r="G28" s="36" t="s">
+      <c r="G28" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="H28" s="36" t="s">
+      <c r="H28" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="I28" s="25">
+      <c r="I28" s="24">
         <f>SUM(I20:I27)</f>
         <v>0</v>
       </c>
       <c r="J28" s="2"/>
     </row>
     <row r="29" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="60" t="s">
+      <c r="A29" s="57" t="s">
         <v>33</v>
       </c>
-      <c r="B29" s="61"/>
-      <c r="C29" s="61"/>
-      <c r="D29" s="61"/>
-      <c r="E29" s="61"/>
-      <c r="F29" s="61"/>
-      <c r="G29" s="61"/>
-      <c r="H29" s="61"/>
-      <c r="I29" s="61"/>
-      <c r="J29" s="7"/>
+      <c r="B29" s="58"/>
+      <c r="C29" s="58"/>
+      <c r="D29" s="58"/>
+      <c r="E29" s="58"/>
+      <c r="F29" s="58"/>
+      <c r="G29" s="58"/>
+      <c r="H29" s="58"/>
+      <c r="I29" s="58"/>
+      <c r="J29" s="6"/>
     </row>
     <row r="30" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="21"/>
-      <c r="B30" s="21"/>
-      <c r="C30" s="21"/>
-      <c r="D30" s="21"/>
-      <c r="E30" s="21"/>
-      <c r="F30" s="21"/>
-      <c r="G30" s="21"/>
-      <c r="H30" s="21"/>
-      <c r="I30" s="21"/>
-      <c r="J30" s="7"/>
+      <c r="A30" s="20"/>
+      <c r="B30" s="20"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
+      <c r="F30" s="20"/>
+      <c r="G30" s="20"/>
+      <c r="H30" s="20"/>
+      <c r="I30" s="20"/>
+      <c r="J30" s="6"/>
     </row>
     <row r="31" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="80" t="s">
+      <c r="A31" s="77" t="s">
         <v>34</v>
       </c>
-      <c r="B31" s="48"/>
-      <c r="C31" s="48"/>
-      <c r="D31" s="48"/>
-      <c r="E31" s="21"/>
-      <c r="F31" s="21"/>
-      <c r="G31" s="21"/>
-      <c r="H31" s="21"/>
-      <c r="I31" s="21"/>
-      <c r="J31" s="7"/>
+      <c r="B31" s="45"/>
+      <c r="C31" s="45"/>
+      <c r="D31" s="45"/>
+      <c r="E31" s="20"/>
+      <c r="F31" s="20"/>
+      <c r="G31" s="20"/>
+      <c r="H31" s="20"/>
+      <c r="I31" s="20"/>
+      <c r="J31" s="6"/>
     </row>
     <row r="32" spans="1:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="80" t="s">
+      <c r="A32" s="77" t="s">
         <v>35</v>
       </c>
-      <c r="B32" s="48"/>
-      <c r="C32" s="48"/>
-      <c r="D32" s="48"/>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
-      <c r="G32" s="21"/>
-      <c r="H32" s="21"/>
-      <c r="I32" s="21"/>
-      <c r="J32" s="7"/>
+      <c r="B32" s="45"/>
+      <c r="C32" s="45"/>
+      <c r="D32" s="45"/>
+      <c r="E32" s="20"/>
+      <c r="F32" s="20"/>
+      <c r="G32" s="20"/>
+      <c r="H32" s="20"/>
+      <c r="I32" s="20"/>
+      <c r="J32" s="6"/>
     </row>
     <row r="33" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="81" t="s">
+      <c r="A33" s="78" t="s">
         <v>12</v>
       </c>
-      <c r="B33" s="82"/>
-      <c r="C33" s="82"/>
-      <c r="D33" s="82"/>
-      <c r="E33" s="21"/>
-      <c r="F33" s="21"/>
-      <c r="G33" s="21"/>
-      <c r="H33" s="21"/>
-      <c r="I33" s="21"/>
-      <c r="J33" s="7"/>
+      <c r="B33" s="79"/>
+      <c r="C33" s="79"/>
+      <c r="D33" s="79"/>
+      <c r="E33" s="20"/>
+      <c r="F33" s="20"/>
+      <c r="G33" s="20"/>
+      <c r="H33" s="20"/>
+      <c r="I33" s="20"/>
+      <c r="J33" s="6"/>
     </row>
     <row r="34" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="52" t="s">
+      <c r="A34" s="49" t="s">
         <v>36</v>
       </c>
-      <c r="B34" s="48"/>
-      <c r="C34" s="52">
+      <c r="B34" s="45"/>
+      <c r="C34" s="49">
         <v>8116409</v>
       </c>
-      <c r="D34" s="48"/>
-      <c r="E34" s="8"/>
-      <c r="F34" s="8"/>
-      <c r="G34" s="8"/>
-      <c r="H34" s="8"/>
-      <c r="I34" s="8"/>
-      <c r="J34" s="9"/>
+      <c r="D34" s="45"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="7"/>
+      <c r="G34" s="7"/>
+      <c r="H34" s="7"/>
+      <c r="I34" s="7"/>
+      <c r="J34" s="8"/>
     </row>
     <row r="35" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="52" t="s">
+      <c r="A35" s="49" t="s">
         <v>37</v>
       </c>
-      <c r="B35" s="48"/>
-      <c r="C35" s="90"/>
-      <c r="D35" s="48"/>
-      <c r="E35" s="8"/>
-      <c r="F35" s="8"/>
-      <c r="G35" s="8"/>
-      <c r="H35" s="8"/>
-      <c r="I35" s="8"/>
-      <c r="J35" s="9"/>
+      <c r="B35" s="45"/>
+      <c r="C35" s="87"/>
+      <c r="D35" s="45"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="7"/>
+      <c r="G35" s="7"/>
+      <c r="H35" s="7"/>
+      <c r="I35" s="7"/>
+      <c r="J35" s="8"/>
     </row>
     <row r="36" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="52" t="s">
+      <c r="A36" s="49" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="48"/>
-      <c r="C36" s="80"/>
-      <c r="D36" s="48"/>
-      <c r="E36" s="8"/>
-      <c r="F36" s="8"/>
-      <c r="G36" s="8"/>
-      <c r="H36" s="8"/>
-      <c r="I36" s="8"/>
-      <c r="J36" s="9"/>
+      <c r="B36" s="45"/>
+      <c r="C36" s="77"/>
+      <c r="D36" s="45"/>
+      <c r="E36" s="7"/>
+      <c r="F36" s="7"/>
+      <c r="G36" s="7"/>
+      <c r="H36" s="7"/>
+      <c r="I36" s="7"/>
+      <c r="J36" s="8"/>
     </row>
     <row r="37" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="19"/>
-      <c r="B37" s="19"/>
-      <c r="C37" s="19"/>
-      <c r="D37" s="19"/>
-      <c r="E37" s="8"/>
-      <c r="F37" s="8"/>
-      <c r="G37" s="8"/>
-      <c r="H37" s="8"/>
-      <c r="I37" s="8"/>
-      <c r="J37" s="9"/>
+      <c r="A37" s="18"/>
+      <c r="B37" s="18"/>
+      <c r="C37" s="18"/>
+      <c r="D37" s="18"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="7"/>
+      <c r="H37" s="7"/>
+      <c r="I37" s="7"/>
+      <c r="J37" s="8"/>
     </row>
     <row r="38" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="19"/>
-      <c r="B38" s="19"/>
-      <c r="C38" s="19"/>
-      <c r="D38" s="19"/>
-      <c r="E38" s="8"/>
-      <c r="F38" s="8"/>
-      <c r="G38" s="8"/>
-      <c r="H38" s="8"/>
-      <c r="I38" s="8"/>
-      <c r="J38" s="9"/>
+      <c r="A38" s="18"/>
+      <c r="B38" s="18"/>
+      <c r="C38" s="18"/>
+      <c r="D38" s="18"/>
+      <c r="E38" s="7"/>
+      <c r="F38" s="7"/>
+      <c r="G38" s="7"/>
+      <c r="H38" s="7"/>
+      <c r="I38" s="7"/>
+      <c r="J38" s="8"/>
     </row>
     <row r="39" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="19"/>
-      <c r="B39" s="19"/>
-      <c r="C39" s="19"/>
-      <c r="D39" s="19"/>
-      <c r="E39" s="8"/>
-      <c r="F39" s="8"/>
-      <c r="G39" s="8"/>
-      <c r="H39" s="8"/>
-      <c r="I39" s="8"/>
-      <c r="J39" s="9"/>
+      <c r="A39" s="18"/>
+      <c r="B39" s="18"/>
+      <c r="C39" s="18"/>
+      <c r="D39" s="18"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="7"/>
+      <c r="G39" s="7"/>
+      <c r="H39" s="7"/>
+      <c r="I39" s="7"/>
+      <c r="J39" s="8"/>
     </row>
     <row r="40" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="19"/>
-      <c r="B40" s="19"/>
-      <c r="C40" s="19"/>
-      <c r="D40" s="19"/>
-      <c r="E40" s="8"/>
-      <c r="F40" s="8"/>
-      <c r="G40" s="8"/>
-      <c r="H40" s="8"/>
-      <c r="I40" s="8"/>
-      <c r="J40" s="9"/>
+      <c r="A40" s="18"/>
+      <c r="B40" s="18"/>
+      <c r="C40" s="18"/>
+      <c r="D40" s="18"/>
+      <c r="E40" s="7"/>
+      <c r="F40" s="7"/>
+      <c r="G40" s="7"/>
+      <c r="H40" s="7"/>
+      <c r="I40" s="7"/>
+      <c r="J40" s="8"/>
     </row>
     <row r="41" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="84" t="s">
+      <c r="A41" s="81" t="s">
         <v>39</v>
       </c>
-      <c r="B41" s="48"/>
-      <c r="C41" s="48"/>
-      <c r="D41" s="48"/>
-      <c r="E41" s="48"/>
-      <c r="F41" s="48"/>
-      <c r="G41" s="48"/>
-      <c r="H41" s="48"/>
-      <c r="I41" s="48"/>
-      <c r="J41" s="9"/>
+      <c r="B41" s="45"/>
+      <c r="C41" s="45"/>
+      <c r="D41" s="45"/>
+      <c r="E41" s="45"/>
+      <c r="F41" s="45"/>
+      <c r="G41" s="45"/>
+      <c r="H41" s="45"/>
+      <c r="I41" s="45"/>
+      <c r="J41" s="8"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A42" s="83" t="s">
+      <c r="A42" s="80" t="s">
         <v>40</v>
       </c>
-      <c r="B42" s="48"/>
-      <c r="C42" s="48"/>
-      <c r="D42" s="48"/>
-      <c r="E42" s="48"/>
-      <c r="F42" s="69" t="s">
+      <c r="B42" s="45"/>
+      <c r="C42" s="45"/>
+      <c r="D42" s="45"/>
+      <c r="E42" s="45"/>
+      <c r="F42" s="66" t="s">
         <v>41</v>
       </c>
-      <c r="G42" s="48"/>
-      <c r="H42" s="48"/>
-      <c r="I42" s="48"/>
-      <c r="J42" s="10"/>
+      <c r="G42" s="45"/>
+      <c r="H42" s="45"/>
+      <c r="I42" s="45"/>
+      <c r="J42" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="45">

</xml_diff>